<commit_message>
Automatiza 127 arquivo(s) de processos no backend
</commit_message>
<xml_diff>
--- a/planilhas/LISTA DE PROCESSO PG + ECO HIBRIDO LADO MENOR.xlsx
+++ b/planilhas/LISTA DE PROCESSO PG + ECO HIBRIDO LADO MENOR.xlsx
@@ -323,7 +323,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F141"/>
+  <dimension ref="A1:F140"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="37" customWidth="1" min="1" max="1"/>
@@ -1534,8 +1534,9 @@
           <t>20X20X1,50MM Nest 1</t>
         </is>
       </c>
-      <c r="D43" t="n">
-        <v>0.331</v>
+      <c r="D43">
+        <f>E43/1000</f>
+        <v/>
       </c>
       <c r="E43" t="n">
         <v>331</v>
@@ -1562,8 +1563,9 @@
           <t>20X20X1,50MM Nest 2</t>
         </is>
       </c>
-      <c r="D44" t="n">
-        <v>0.001</v>
+      <c r="D44">
+        <f>E44/1000</f>
+        <v/>
       </c>
       <c r="E44" t="n">
         <v>1</v>
@@ -1590,8 +1592,9 @@
           <t>20X20X1,50MM Nest 3</t>
         </is>
       </c>
-      <c r="D45" t="n">
-        <v>0.001</v>
+      <c r="D45">
+        <f>E45/1000</f>
+        <v/>
       </c>
       <c r="E45" t="n">
         <v>1</v>
@@ -1618,8 +1621,9 @@
           <t>20X20X1,50MM Nest 4</t>
         </is>
       </c>
-      <c r="D46" t="n">
-        <v>0.332</v>
+      <c r="D46">
+        <f>E46/1000</f>
+        <v/>
       </c>
       <c r="E46" t="n">
         <v>332</v>
@@ -1646,8 +1650,9 @@
           <t>20X20X1,50MM Nest 5</t>
         </is>
       </c>
-      <c r="D47" t="n">
-        <v>0.332</v>
+      <c r="D47">
+        <f>E47/1000</f>
+        <v/>
       </c>
       <c r="E47" t="n">
         <v>332</v>
@@ -1674,8 +1679,9 @@
           <t>20X20X1,50MM Nest 6</t>
         </is>
       </c>
-      <c r="D48" t="n">
-        <v>0.332</v>
+      <c r="D48">
+        <f>E48/1000</f>
+        <v/>
       </c>
       <c r="E48" t="n">
         <v>332</v>
@@ -1702,8 +1708,9 @@
           <t>20X20X1,50MM Nest 7</t>
         </is>
       </c>
-      <c r="D49" t="n">
-        <v>0.001</v>
+      <c r="D49">
+        <f>E49/1000</f>
+        <v/>
       </c>
       <c r="E49" t="n">
         <v>1</v>
@@ -2485,7 +2492,7 @@
         </is>
       </c>
       <c r="D76">
-        <f>E76/1700</f>
+        <f>E76/1000</f>
         <v/>
       </c>
       <c r="E76" t="n">
@@ -2514,11 +2521,11 @@
         </is>
       </c>
       <c r="D77">
-        <f>E77/1700</f>
+        <f>E77/1000</f>
         <v/>
       </c>
       <c r="E77" t="n">
-        <v>130</v>
+        <v>99</v>
       </c>
       <c r="F77" s="1" t="inlineStr">
         <is>
@@ -2543,11 +2550,11 @@
         </is>
       </c>
       <c r="D78">
-        <f>E78/1700</f>
+        <f>E78/1000</f>
         <v/>
       </c>
       <c r="E78" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F78" s="1" t="inlineStr">
         <is>
@@ -2572,11 +2579,11 @@
         </is>
       </c>
       <c r="D79">
-        <f>E79/1700</f>
+        <f>E79/1000</f>
         <v/>
       </c>
       <c r="E79" t="n">
-        <v>202</v>
+        <v>219</v>
       </c>
       <c r="F79" s="1" t="inlineStr">
         <is>
@@ -2601,11 +2608,11 @@
         </is>
       </c>
       <c r="D80">
-        <f>E80/1700</f>
+        <f>E80/1000</f>
         <v/>
       </c>
       <c r="E80" t="n">
-        <v>16</v>
+        <v>1</v>
       </c>
       <c r="F80" s="1" t="inlineStr">
         <is>
@@ -2630,7 +2637,7 @@
         </is>
       </c>
       <c r="D81">
-        <f>E81/1700</f>
+        <f>E81/1000</f>
         <v/>
       </c>
       <c r="E81" t="n">
@@ -2659,11 +2666,11 @@
         </is>
       </c>
       <c r="D82">
-        <f>E82/1700</f>
+        <f>E82/1000</f>
         <v/>
       </c>
       <c r="E82" t="n">
-        <v>221</v>
+        <v>5</v>
       </c>
       <c r="F82" s="1" t="inlineStr">
         <is>
@@ -2688,7 +2695,7 @@
         </is>
       </c>
       <c r="D83">
-        <f>E83/1700</f>
+        <f>E83/1000</f>
         <v/>
       </c>
       <c r="E83" t="n">
@@ -2708,24 +2715,23 @@
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>Laser Chapa</t>
+          <t>Serra</t>
         </is>
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>2,65 Nest 9</t>
-        </is>
-      </c>
-      <c r="D84">
-        <f>E84/1700</f>
-        <v/>
+          <t>Tubo Bdj 433 MM</t>
+        </is>
+      </c>
+      <c r="D84" t="n">
+        <v>5</v>
       </c>
       <c r="E84" t="n">
-        <v>1</v>
+        <v>5000</v>
       </c>
       <c r="F84" s="1" t="inlineStr">
         <is>
-          <t>000345</t>
+          <t>000379</t>
         </is>
       </c>
     </row>
@@ -2742,7 +2748,7 @@
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>Tubo Bdj 433 MM</t>
+          <t>Tubo Bdj 493 MM</t>
         </is>
       </c>
       <c r="D85" t="n">
@@ -2753,7 +2759,7 @@
       </c>
       <c r="F85" s="1" t="inlineStr">
         <is>
-          <t>000379</t>
+          <t>000380</t>
         </is>
       </c>
     </row>
@@ -2765,23 +2771,23 @@
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>Serra</t>
+          <t>Dobradeira de Arames</t>
         </is>
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>Tubo Bdj 493 MM</t>
+          <t>Arame Toldo Lateral</t>
         </is>
       </c>
       <c r="D86" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="E86" t="n">
-        <v>5000</v>
+        <v>2000</v>
       </c>
       <c r="F86" s="1" t="inlineStr">
         <is>
-          <t>000380</t>
+          <t>001439</t>
         </is>
       </c>
     </row>
@@ -2798,18 +2804,18 @@
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>Arame Toldo Lateral</t>
+          <t>Arame Toldo Trecho Reto</t>
         </is>
       </c>
       <c r="D87" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E87" t="n">
-        <v>2000</v>
+        <v>3000</v>
       </c>
       <c r="F87" s="1" t="inlineStr">
         <is>
-          <t>001439</t>
+          <t>001440</t>
         </is>
       </c>
     </row>
@@ -2821,23 +2827,23 @@
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>Dobradeira de Arames</t>
+          <t>Dobradeira de Chapas</t>
         </is>
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>Arame Toldo Trecho Reto</t>
+          <t>J 1732 mm</t>
         </is>
       </c>
       <c r="D88" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E88" t="n">
-        <v>3000</v>
+        <v>4000</v>
       </c>
       <c r="F88" s="1" t="inlineStr">
         <is>
-          <t>001440</t>
+          <t>000346</t>
         </is>
       </c>
     </row>
@@ -2854,18 +2860,18 @@
       </c>
       <c r="C89" t="inlineStr">
         <is>
-          <t>J 1732 mm</t>
+          <t>J 333 mm</t>
         </is>
       </c>
       <c r="D89" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="E89" t="n">
-        <v>4000</v>
+        <v>2000</v>
       </c>
       <c r="F89" s="1" t="inlineStr">
         <is>
-          <t>000346</t>
+          <t>000347</t>
         </is>
       </c>
     </row>
@@ -2882,18 +2888,18 @@
       </c>
       <c r="C90" t="inlineStr">
         <is>
-          <t>J 333 mm</t>
+          <t>J 1028 mm</t>
         </is>
       </c>
       <c r="D90" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E90" t="n">
-        <v>2000</v>
+        <v>1000</v>
       </c>
       <c r="F90" s="1" t="inlineStr">
         <is>
-          <t>000347</t>
+          <t>000348</t>
         </is>
       </c>
     </row>
@@ -2910,7 +2916,7 @@
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>J 1028 mm</t>
+          <t>Fechamento Saia</t>
         </is>
       </c>
       <c r="D91" t="n">
@@ -2921,7 +2927,7 @@
       </c>
       <c r="F91" s="1" t="inlineStr">
         <is>
-          <t>000348</t>
+          <t>000349</t>
         </is>
       </c>
     </row>
@@ -2938,7 +2944,7 @@
       </c>
       <c r="C92" t="inlineStr">
         <is>
-          <t>Fechamento Saia</t>
+          <t>Fechamento Parachoque Móvel</t>
         </is>
       </c>
       <c r="D92" t="n">
@@ -2949,7 +2955,7 @@
       </c>
       <c r="F92" s="1" t="inlineStr">
         <is>
-          <t>000349</t>
+          <t>000350</t>
         </is>
       </c>
     </row>
@@ -2966,7 +2972,7 @@
       </c>
       <c r="C93" t="inlineStr">
         <is>
-          <t>Fechamento Parachoque Móvel</t>
+          <t>Chapa Frontal Testeira</t>
         </is>
       </c>
       <c r="D93" t="n">
@@ -2977,7 +2983,7 @@
       </c>
       <c r="F93" s="1" t="inlineStr">
         <is>
-          <t>000350</t>
+          <t>000351</t>
         </is>
       </c>
     </row>
@@ -2994,7 +3000,7 @@
       </c>
       <c r="C94" t="inlineStr">
         <is>
-          <t>Chapa Frontal Testeira</t>
+          <t>Chapa Central Fixação Toldo</t>
         </is>
       </c>
       <c r="D94" t="n">
@@ -3005,7 +3011,7 @@
       </c>
       <c r="F94" s="1" t="inlineStr">
         <is>
-          <t>000351</t>
+          <t>000352</t>
         </is>
       </c>
     </row>
@@ -3022,18 +3028,18 @@
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>Chapa Central Fixação Toldo</t>
+          <t>Encaixe Parachoque Direito</t>
         </is>
       </c>
       <c r="D95" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="E95" t="n">
-        <v>1000</v>
+        <v>3000</v>
       </c>
       <c r="F95" s="1" t="inlineStr">
         <is>
-          <t>000352</t>
+          <t>000353</t>
         </is>
       </c>
     </row>
@@ -3050,18 +3056,18 @@
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t>Encaixe Parachoque Direito</t>
+          <t>Encaixe Parachoque Esquerda</t>
         </is>
       </c>
       <c r="D96" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E96" t="n">
-        <v>3000</v>
+        <v>2000</v>
       </c>
       <c r="F96" s="1" t="inlineStr">
         <is>
-          <t>000353</t>
+          <t>000354</t>
         </is>
       </c>
     </row>
@@ -3078,18 +3084,18 @@
       </c>
       <c r="C97" t="inlineStr">
         <is>
-          <t>Encaixe Parachoque Esquerda</t>
+          <t>Bdj Esquerda Amassamento</t>
         </is>
       </c>
       <c r="D97" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="E97" t="n">
-        <v>2000</v>
+        <v>4000</v>
       </c>
       <c r="F97" s="1" t="inlineStr">
         <is>
-          <t>000354</t>
+          <t>000355</t>
         </is>
       </c>
     </row>
@@ -3106,7 +3112,7 @@
       </c>
       <c r="C98" t="inlineStr">
         <is>
-          <t>Bdj Esquerda Amassamento</t>
+          <t>Bdj Esquerda Dobra</t>
         </is>
       </c>
       <c r="D98" t="n">
@@ -3117,7 +3123,7 @@
       </c>
       <c r="F98" s="1" t="inlineStr">
         <is>
-          <t>000355</t>
+          <t>000356</t>
         </is>
       </c>
     </row>
@@ -3134,7 +3140,7 @@
       </c>
       <c r="C99" t="inlineStr">
         <is>
-          <t>Bdj Esquerda Dobra</t>
+          <t>Bdj Direita Amassamento</t>
         </is>
       </c>
       <c r="D99" t="n">
@@ -3145,7 +3151,7 @@
       </c>
       <c r="F99" s="1" t="inlineStr">
         <is>
-          <t>000356</t>
+          <t>000357</t>
         </is>
       </c>
     </row>
@@ -3162,7 +3168,7 @@
       </c>
       <c r="C100" t="inlineStr">
         <is>
-          <t>Bdj Direita Amassamento</t>
+          <t>Bdj Direita Dobra</t>
         </is>
       </c>
       <c r="D100" t="n">
@@ -3173,7 +3179,7 @@
       </c>
       <c r="F100" s="1" t="inlineStr">
         <is>
-          <t>000357</t>
+          <t>000358</t>
         </is>
       </c>
     </row>
@@ -3190,18 +3196,18 @@
       </c>
       <c r="C101" t="inlineStr">
         <is>
-          <t>Bdj Direita Dobra</t>
+          <t>Bdj Esquerda Base Amassamento</t>
         </is>
       </c>
       <c r="D101" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="E101" t="n">
-        <v>4000</v>
+        <v>1000</v>
       </c>
       <c r="F101" s="1" t="inlineStr">
         <is>
-          <t>000358</t>
+          <t>000359</t>
         </is>
       </c>
     </row>
@@ -3218,7 +3224,7 @@
       </c>
       <c r="C102" t="inlineStr">
         <is>
-          <t>Bdj Esquerda Base Amassamento</t>
+          <t>Bdj Esquerda Base Dobra</t>
         </is>
       </c>
       <c r="D102" t="n">
@@ -3229,7 +3235,7 @@
       </c>
       <c r="F102" s="1" t="inlineStr">
         <is>
-          <t>000359</t>
+          <t>000360</t>
         </is>
       </c>
     </row>
@@ -3246,7 +3252,7 @@
       </c>
       <c r="C103" t="inlineStr">
         <is>
-          <t>Bdj Esquerda Base Dobra</t>
+          <t>Bdj Direita Base Amassamento</t>
         </is>
       </c>
       <c r="D103" t="n">
@@ -3257,7 +3263,7 @@
       </c>
       <c r="F103" s="1" t="inlineStr">
         <is>
-          <t>000360</t>
+          <t>000361</t>
         </is>
       </c>
     </row>
@@ -3274,7 +3280,7 @@
       </c>
       <c r="C104" t="inlineStr">
         <is>
-          <t>Bdj Direita Base Amassamento</t>
+          <t>Bdj Direita Base Dobra</t>
         </is>
       </c>
       <c r="D104" t="n">
@@ -3285,7 +3291,7 @@
       </c>
       <c r="F104" s="1" t="inlineStr">
         <is>
-          <t>000361</t>
+          <t>000362</t>
         </is>
       </c>
     </row>
@@ -3302,18 +3308,18 @@
       </c>
       <c r="C105" t="inlineStr">
         <is>
-          <t>Bdj Direita Base Dobra</t>
+          <t>Chapa Gancho Pallet</t>
         </is>
       </c>
       <c r="D105" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E105" t="n">
         <v>1000</v>
       </c>
       <c r="F105" s="1" t="inlineStr">
         <is>
-          <t>000362</t>
+          <t>000363</t>
         </is>
       </c>
     </row>
@@ -3325,23 +3331,23 @@
       </c>
       <c r="B106" t="inlineStr">
         <is>
-          <t>Dobradeira de Chapas</t>
+          <t>Solda Mig</t>
         </is>
       </c>
       <c r="C106" t="inlineStr">
         <is>
-          <t>Chapa Gancho Pallet</t>
+          <t>Lateral Esquerda Tubular</t>
         </is>
       </c>
       <c r="D106" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E106" t="n">
         <v>1000</v>
       </c>
       <c r="F106" s="1" t="inlineStr">
         <is>
-          <t>000363</t>
+          <t>000364</t>
         </is>
       </c>
     </row>
@@ -3358,7 +3364,7 @@
       </c>
       <c r="C107" t="inlineStr">
         <is>
-          <t>Lateral Esquerda Tubular</t>
+          <t>Lateral Direita Tubular</t>
         </is>
       </c>
       <c r="D107" t="n">
@@ -3369,7 +3375,7 @@
       </c>
       <c r="F107" s="1" t="inlineStr">
         <is>
-          <t>000364</t>
+          <t>000365</t>
         </is>
       </c>
     </row>
@@ -3386,7 +3392,7 @@
       </c>
       <c r="C108" t="inlineStr">
         <is>
-          <t>Lateral Direita Tubular</t>
+          <t>Lateral Esquerda Chaparia + Triângulo 2,65</t>
         </is>
       </c>
       <c r="D108" t="n">
@@ -3397,7 +3403,7 @@
       </c>
       <c r="F108" s="1" t="inlineStr">
         <is>
-          <t>000365</t>
+          <t>000366</t>
         </is>
       </c>
     </row>
@@ -3414,7 +3420,7 @@
       </c>
       <c r="C109" t="inlineStr">
         <is>
-          <t>Lateral Esquerda Chaparia + Triângulo 2,65</t>
+          <t>Lateral Direita Chaparia + Triângulo 2,65</t>
         </is>
       </c>
       <c r="D109" t="n">
@@ -3425,7 +3431,7 @@
       </c>
       <c r="F109" s="1" t="inlineStr">
         <is>
-          <t>000366</t>
+          <t>000367</t>
         </is>
       </c>
     </row>
@@ -3442,7 +3448,7 @@
       </c>
       <c r="C110" t="inlineStr">
         <is>
-          <t>Lateral Direita Chaparia + Triângulo 2,65</t>
+          <t>Lateral Esquerda Arruela Quadrada 2,65</t>
         </is>
       </c>
       <c r="D110" t="n">
@@ -3453,7 +3459,7 @@
       </c>
       <c r="F110" s="1" t="inlineStr">
         <is>
-          <t>000367</t>
+          <t>000368</t>
         </is>
       </c>
     </row>
@@ -3470,7 +3476,7 @@
       </c>
       <c r="C111" t="inlineStr">
         <is>
-          <t>Lateral Esquerda Arruela Quadrada 2,65</t>
+          <t>Lateral Direita Arruela Quadrada 2,65</t>
         </is>
       </c>
       <c r="D111" t="n">
@@ -3481,7 +3487,7 @@
       </c>
       <c r="F111" s="1" t="inlineStr">
         <is>
-          <t>000368</t>
+          <t>000369</t>
         </is>
       </c>
     </row>
@@ -3498,7 +3504,7 @@
       </c>
       <c r="C112" t="inlineStr">
         <is>
-          <t>Lateral Direita Arruela Quadrada 2,65</t>
+          <t>Quadro Cremalheira</t>
         </is>
       </c>
       <c r="D112" t="n">
@@ -3509,7 +3515,7 @@
       </c>
       <c r="F112" s="1" t="inlineStr">
         <is>
-          <t>000369</t>
+          <t>000386</t>
         </is>
       </c>
     </row>
@@ -3526,7 +3532,7 @@
       </c>
       <c r="C113" t="inlineStr">
         <is>
-          <t>Quadro Cremalheira</t>
+          <t>Levantamento Corpo</t>
         </is>
       </c>
       <c r="D113" t="n">
@@ -3537,7 +3543,7 @@
       </c>
       <c r="F113" s="1" t="inlineStr">
         <is>
-          <t>000386</t>
+          <t>000370</t>
         </is>
       </c>
     </row>
@@ -3554,7 +3560,7 @@
       </c>
       <c r="C114" t="inlineStr">
         <is>
-          <t>Levantamento Corpo</t>
+          <t>Chaparia Testeira + Saia + Canaletas</t>
         </is>
       </c>
       <c r="D114" t="n">
@@ -3565,7 +3571,7 @@
       </c>
       <c r="F114" s="1" t="inlineStr">
         <is>
-          <t>000370</t>
+          <t>000371</t>
         </is>
       </c>
     </row>
@@ -3582,18 +3588,18 @@
       </c>
       <c r="C115" t="inlineStr">
         <is>
-          <t>Chaparia Testeira + Saia + Canaletas</t>
+          <t>Bdj Esquerda Tubo + Mão francesa (inferior)</t>
         </is>
       </c>
       <c r="D115" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="E115" t="n">
-        <v>1000</v>
+        <v>4000</v>
       </c>
       <c r="F115" s="1" t="inlineStr">
         <is>
-          <t>000371</t>
+          <t>001441</t>
         </is>
       </c>
     </row>
@@ -3610,7 +3616,7 @@
       </c>
       <c r="C116" t="inlineStr">
         <is>
-          <t>Bdj Esquerda Tubo + Mão francesa (inferior)</t>
+          <t>Bdj Direita Tubo + Mão francesa (inferior)</t>
         </is>
       </c>
       <c r="D116" t="n">
@@ -3621,7 +3627,7 @@
       </c>
       <c r="F116" s="1" t="inlineStr">
         <is>
-          <t>001441</t>
+          <t>001442</t>
         </is>
       </c>
     </row>
@@ -3638,18 +3644,18 @@
       </c>
       <c r="C117" t="inlineStr">
         <is>
-          <t>Bdj Direita Tubo + Mão francesa (inferior)</t>
+          <t>Bdj Esquerda Base Tubo + Mão francesa (inferior)</t>
         </is>
       </c>
       <c r="D117" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="E117" t="n">
-        <v>4000</v>
+        <v>1000</v>
       </c>
       <c r="F117" s="1" t="inlineStr">
         <is>
-          <t>001442</t>
+          <t>001443</t>
         </is>
       </c>
     </row>
@@ -3666,7 +3672,7 @@
       </c>
       <c r="C118" t="inlineStr">
         <is>
-          <t>Bdj Esquerda Base Tubo + Mão francesa (inferior)</t>
+          <t>Bdj Direita Base Tubo + Mão francesa (inferior)</t>
         </is>
       </c>
       <c r="D118" t="n">
@@ -3677,7 +3683,7 @@
       </c>
       <c r="F118" s="1" t="inlineStr">
         <is>
-          <t>001443</t>
+          <t>001444</t>
         </is>
       </c>
     </row>
@@ -3694,18 +3700,18 @@
       </c>
       <c r="C119" t="inlineStr">
         <is>
-          <t>Bdj Direita Base Tubo + Mão francesa (inferior)</t>
+          <t>Bdj Esquerda Tubo + Mão francesa (superior)</t>
         </is>
       </c>
       <c r="D119" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="E119" t="n">
-        <v>1000</v>
+        <v>4000</v>
       </c>
       <c r="F119" s="1" t="inlineStr">
         <is>
-          <t>001444</t>
+          <t>001445</t>
         </is>
       </c>
     </row>
@@ -3722,7 +3728,7 @@
       </c>
       <c r="C120" t="inlineStr">
         <is>
-          <t>Bdj Esquerda Tubo + Mão francesa (superior)</t>
+          <t>Bdj Direita Tubo + Mão francesa (superior)</t>
         </is>
       </c>
       <c r="D120" t="n">
@@ -3733,7 +3739,7 @@
       </c>
       <c r="F120" s="1" t="inlineStr">
         <is>
-          <t>001445</t>
+          <t>001446</t>
         </is>
       </c>
     </row>
@@ -3750,18 +3756,18 @@
       </c>
       <c r="C121" t="inlineStr">
         <is>
-          <t>Bdj Direita Tubo + Mão francesa (superior)</t>
+          <t>Bdj Esquerda Base Tubo + Mão francesa (superior)</t>
         </is>
       </c>
       <c r="D121" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="E121" t="n">
-        <v>4000</v>
+        <v>1000</v>
       </c>
       <c r="F121" s="1" t="inlineStr">
         <is>
-          <t>001446</t>
+          <t>001447</t>
         </is>
       </c>
     </row>
@@ -3778,7 +3784,7 @@
       </c>
       <c r="C122" t="inlineStr">
         <is>
-          <t>Bdj Esquerda Base Tubo + Mão francesa (superior)</t>
+          <t>Bdj Direita Base Tubo + Mão francesa (superior)</t>
         </is>
       </c>
       <c r="D122" t="n">
@@ -3789,7 +3795,7 @@
       </c>
       <c r="F122" s="1" t="inlineStr">
         <is>
-          <t>001447</t>
+          <t>001448</t>
         </is>
       </c>
     </row>
@@ -3806,7 +3812,7 @@
       </c>
       <c r="C123" t="inlineStr">
         <is>
-          <t>Bdj Direita Base Tubo + Mão francesa (superior)</t>
+          <t>Aramado Toldo</t>
         </is>
       </c>
       <c r="D123" t="n">
@@ -3817,7 +3823,7 @@
       </c>
       <c r="F123" s="1" t="inlineStr">
         <is>
-          <t>001448</t>
+          <t>000376</t>
         </is>
       </c>
     </row>
@@ -3834,7 +3840,7 @@
       </c>
       <c r="C124" t="inlineStr">
         <is>
-          <t>Aramado Toldo</t>
+          <t>Aramado Toldo + Chapa Fixação</t>
         </is>
       </c>
       <c r="D124" t="n">
@@ -3845,7 +3851,7 @@
       </c>
       <c r="F124" s="1" t="inlineStr">
         <is>
-          <t>000376</t>
+          <t>000377</t>
         </is>
       </c>
     </row>
@@ -3862,7 +3868,7 @@
       </c>
       <c r="C125" t="inlineStr">
         <is>
-          <t>Aramado Toldo + Chapa Fixação</t>
+          <t>Parachoque + Chapa 2,65</t>
         </is>
       </c>
       <c r="D125" t="n">
@@ -3873,37 +3879,12 @@
       </c>
       <c r="F125" s="1" t="inlineStr">
         <is>
-          <t>000377</t>
+          <t>000378</t>
         </is>
       </c>
     </row>
     <row r="126">
-      <c r="A126" t="inlineStr">
-        <is>
-          <t>PG + ECONOMIA HIBRIDO</t>
-        </is>
-      </c>
-      <c r="B126" t="inlineStr">
-        <is>
-          <t>Solda Mig</t>
-        </is>
-      </c>
-      <c r="C126" t="inlineStr">
-        <is>
-          <t>Parachoque + Chapa 2,65</t>
-        </is>
-      </c>
-      <c r="D126" t="n">
-        <v>1</v>
-      </c>
-      <c r="E126" t="n">
-        <v>1000</v>
-      </c>
-      <c r="F126" s="1" t="inlineStr">
-        <is>
-          <t>000378</t>
-        </is>
-      </c>
+      <c r="F126" s="1" t="n"/>
     </row>
     <row r="127">
       <c r="F127" s="1" t="n"/>
@@ -3946,9 +3927,6 @@
     </row>
     <row r="140">
       <c r="F140" s="1" t="n"/>
-    </row>
-    <row r="141">
-      <c r="F141" s="1" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Automatiza 134 arquivo(s) de processos no backend
</commit_message>
<xml_diff>
--- a/planilhas/LISTA DE PROCESSO PG + ECO HIBRIDO LADO MENOR.xlsx
+++ b/planilhas/LISTA DE PROCESSO PG + ECO HIBRIDO LADO MENOR.xlsx
@@ -16,11 +16,15 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="1">
+  <fonts count="2">
     <font>
       <name val="Calibri"/>
       <color theme="1"/>
       <sz val="11"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <sz val="8"/>
     </font>
   </fonts>
   <fills count="2">
@@ -323,7 +327,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F140"/>
+  <dimension ref="A1:F128"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="37" customWidth="1" min="1" max="1"/>
@@ -383,11 +387,11 @@
         </is>
       </c>
       <c r="D2">
-        <f>E2/1700</f>
+        <f>E2/100</f>
         <v/>
       </c>
       <c r="E2" t="n">
-        <v>187</v>
+        <v>94</v>
       </c>
       <c r="F2" s="1" t="inlineStr">
         <is>
@@ -412,11 +416,11 @@
         </is>
       </c>
       <c r="D3">
-        <f>E3/1700</f>
+        <f>E3/100</f>
         <v/>
       </c>
       <c r="E3" t="n">
-        <v>1212</v>
+        <v>713</v>
       </c>
       <c r="F3" s="1" t="inlineStr">
         <is>
@@ -441,7 +445,7 @@
         </is>
       </c>
       <c r="D4">
-        <f>E4/1700</f>
+        <f>E4/100</f>
         <v/>
       </c>
       <c r="E4" t="n">
@@ -466,19 +470,19 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>15X15 Nest 4</t>
+          <t>20X20X0,9MM Nest 1</t>
         </is>
       </c>
       <c r="D5">
-        <f>E5/1700</f>
+        <f>E5/100</f>
         <v/>
       </c>
       <c r="E5" t="n">
-        <v>1</v>
+        <v>177</v>
       </c>
       <c r="F5" s="1" t="inlineStr">
         <is>
-          <t>000273</t>
+          <t>001395</t>
         </is>
       </c>
     </row>
@@ -495,18 +499,19 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>20X20X0,9MM Nest 1</t>
-        </is>
-      </c>
-      <c r="D6" t="n">
-        <v>1</v>
+          <t>20X20X0,9MM Nest 2</t>
+        </is>
+      </c>
+      <c r="D6">
+        <f>E6/100</f>
+        <v/>
       </c>
       <c r="E6" t="n">
-        <v>1000</v>
+        <v>60</v>
       </c>
       <c r="F6" s="1" t="inlineStr">
         <is>
-          <t>001395</t>
+          <t>001396</t>
         </is>
       </c>
     </row>
@@ -523,18 +528,19 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>20X20X0,9MM Nest 2</t>
-        </is>
-      </c>
-      <c r="D7" t="n">
-        <v>1</v>
+          <t>20X20X0,9MM Nest 3</t>
+        </is>
+      </c>
+      <c r="D7">
+        <f>E7/100</f>
+        <v/>
       </c>
       <c r="E7" t="n">
-        <v>1000</v>
+        <v>201</v>
       </c>
       <c r="F7" s="1" t="inlineStr">
         <is>
-          <t>001396</t>
+          <t>001397</t>
         </is>
       </c>
     </row>
@@ -551,18 +557,19 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>20X20X0,9MM Nest 3</t>
-        </is>
-      </c>
-      <c r="D8" t="n">
-        <v>1</v>
+          <t>20X20X0,9MM Nest 4</t>
+        </is>
+      </c>
+      <c r="D8">
+        <f>E8/100</f>
+        <v/>
       </c>
       <c r="E8" t="n">
-        <v>1000</v>
+        <v>118</v>
       </c>
       <c r="F8" s="1" t="inlineStr">
         <is>
-          <t>001397</t>
+          <t>001398</t>
         </is>
       </c>
     </row>
@@ -579,18 +586,19 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>20X20X0,9MM Nest 4</t>
-        </is>
-      </c>
-      <c r="D9" t="n">
-        <v>1</v>
+          <t>20X20X0,9MM Nest 5</t>
+        </is>
+      </c>
+      <c r="D9">
+        <f>E9/100</f>
+        <v/>
       </c>
       <c r="E9" t="n">
-        <v>1000</v>
+        <v>158</v>
       </c>
       <c r="F9" s="1" t="inlineStr">
         <is>
-          <t>001398</t>
+          <t>001399</t>
         </is>
       </c>
     </row>
@@ -607,18 +615,19 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>20X20X0,9MM Nest 5</t>
-        </is>
-      </c>
-      <c r="D10" t="n">
-        <v>1</v>
+          <t>20X20X0,9MM Nest 6</t>
+        </is>
+      </c>
+      <c r="D10">
+        <f>E10/100</f>
+        <v/>
       </c>
       <c r="E10" t="n">
-        <v>1000</v>
+        <v>366</v>
       </c>
       <c r="F10" s="1" t="inlineStr">
         <is>
-          <t>001399</t>
+          <t>001400</t>
         </is>
       </c>
     </row>
@@ -635,18 +644,19 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>20X20X0,9MM Nest 6</t>
-        </is>
-      </c>
-      <c r="D11" t="n">
-        <v>1</v>
+          <t>20X20X0,9MM Nest 7</t>
+        </is>
+      </c>
+      <c r="D11">
+        <f>E11/100</f>
+        <v/>
       </c>
       <c r="E11" t="n">
-        <v>1000</v>
+        <v>499</v>
       </c>
       <c r="F11" s="1" t="inlineStr">
         <is>
-          <t>001400</t>
+          <t>001401</t>
         </is>
       </c>
     </row>
@@ -663,18 +673,19 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>20X20X0,9MM Nest 7</t>
-        </is>
-      </c>
-      <c r="D12" t="n">
-        <v>1</v>
+          <t>20X20X0,9MM Nest 8</t>
+        </is>
+      </c>
+      <c r="D12">
+        <f>E12/100</f>
+        <v/>
       </c>
       <c r="E12" t="n">
-        <v>1000</v>
+        <v>599</v>
       </c>
       <c r="F12" s="1" t="inlineStr">
         <is>
-          <t>001401</t>
+          <t>001402</t>
         </is>
       </c>
     </row>
@@ -691,18 +702,19 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>20X20X0,9MM Nest 8</t>
-        </is>
-      </c>
-      <c r="D13" t="n">
-        <v>1</v>
+          <t>20X20X0,9MM Nest 9</t>
+        </is>
+      </c>
+      <c r="D13">
+        <f>E13/100</f>
+        <v/>
       </c>
       <c r="E13" t="n">
-        <v>1000</v>
+        <v>98</v>
       </c>
       <c r="F13" s="1" t="inlineStr">
         <is>
-          <t>001402</t>
+          <t>001403</t>
         </is>
       </c>
     </row>
@@ -719,18 +731,19 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>20X20X0,9MM Nest 9</t>
-        </is>
-      </c>
-      <c r="D14" t="n">
-        <v>1</v>
+          <t>20X20X0,9MM Nest 10</t>
+        </is>
+      </c>
+      <c r="D14">
+        <f>E14/100</f>
+        <v/>
       </c>
       <c r="E14" t="n">
-        <v>1000</v>
+        <v>200</v>
       </c>
       <c r="F14" s="1" t="inlineStr">
         <is>
-          <t>001403</t>
+          <t>001404</t>
         </is>
       </c>
     </row>
@@ -747,18 +760,19 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>20X20X0,9MM Nest 10</t>
-        </is>
-      </c>
-      <c r="D15" t="n">
-        <v>1</v>
+          <t>20X20X0,9MM Nest 11</t>
+        </is>
+      </c>
+      <c r="D15">
+        <f>E15/100</f>
+        <v/>
       </c>
       <c r="E15" t="n">
-        <v>1000</v>
+        <v>33</v>
       </c>
       <c r="F15" s="1" t="inlineStr">
         <is>
-          <t>001404</t>
+          <t>001405</t>
         </is>
       </c>
     </row>
@@ -775,18 +789,19 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>20X20X0,9MM Nest 11</t>
-        </is>
-      </c>
-      <c r="D16" t="n">
-        <v>1</v>
+          <t>20X20X0,9MM Nest 12</t>
+        </is>
+      </c>
+      <c r="D16">
+        <f>E16/100</f>
+        <v/>
       </c>
       <c r="E16" t="n">
-        <v>1000</v>
+        <v>90</v>
       </c>
       <c r="F16" s="1" t="inlineStr">
         <is>
-          <t>001405</t>
+          <t>001406</t>
         </is>
       </c>
     </row>
@@ -803,18 +818,19 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>20X20X0,9MM Nest 12</t>
-        </is>
-      </c>
-      <c r="D17" t="n">
-        <v>1</v>
+          <t>20X20X0,9MM Nest 13</t>
+        </is>
+      </c>
+      <c r="D17">
+        <f>E17/100</f>
+        <v/>
       </c>
       <c r="E17" t="n">
-        <v>1000</v>
+        <v>133</v>
       </c>
       <c r="F17" s="1" t="inlineStr">
         <is>
-          <t>001406</t>
+          <t>001407</t>
         </is>
       </c>
     </row>
@@ -831,18 +847,19 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>20X20X0,9MM Nest 13</t>
-        </is>
-      </c>
-      <c r="D18" t="n">
-        <v>1</v>
+          <t>20X20X0,9MM Nest 14</t>
+        </is>
+      </c>
+      <c r="D18">
+        <f>E18/100</f>
+        <v/>
       </c>
       <c r="E18" t="n">
-        <v>1000</v>
+        <v>732</v>
       </c>
       <c r="F18" s="1" t="inlineStr">
         <is>
-          <t>001407</t>
+          <t>001408</t>
         </is>
       </c>
     </row>
@@ -859,18 +876,19 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>20X20X0,9MM Nest 14</t>
-        </is>
-      </c>
-      <c r="D19" t="n">
-        <v>1</v>
+          <t>20X20X0,9MM Nest 15</t>
+        </is>
+      </c>
+      <c r="D19">
+        <f>E19/100</f>
+        <v/>
       </c>
       <c r="E19" t="n">
-        <v>1000</v>
+        <v>266</v>
       </c>
       <c r="F19" s="1" t="inlineStr">
         <is>
-          <t>001408</t>
+          <t>001409</t>
         </is>
       </c>
     </row>
@@ -887,18 +905,19 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>20X20X0,9MM Nest 15</t>
-        </is>
-      </c>
-      <c r="D20" t="n">
-        <v>1</v>
+          <t>20X20X0,9MM Nest 16</t>
+        </is>
+      </c>
+      <c r="D20">
+        <f>E20/100</f>
+        <v/>
       </c>
       <c r="E20" t="n">
-        <v>1000</v>
+        <v>266</v>
       </c>
       <c r="F20" s="1" t="inlineStr">
         <is>
-          <t>001409</t>
+          <t>001410</t>
         </is>
       </c>
     </row>
@@ -915,18 +934,19 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>20X20X0,9MM Nest 16</t>
-        </is>
-      </c>
-      <c r="D21" t="n">
-        <v>1</v>
+          <t>20X20X0,9MM Nest 17</t>
+        </is>
+      </c>
+      <c r="D21">
+        <f>E21/100</f>
+        <v/>
       </c>
       <c r="E21" t="n">
-        <v>1000</v>
+        <v>5</v>
       </c>
       <c r="F21" s="1" t="inlineStr">
         <is>
-          <t>001410</t>
+          <t>001411</t>
         </is>
       </c>
     </row>
@@ -943,18 +963,19 @@
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>20X20X0,9MM Nest 17</t>
-        </is>
-      </c>
-      <c r="D22" t="n">
-        <v>1</v>
+          <t>20X20X0,9MM Nest 18</t>
+        </is>
+      </c>
+      <c r="D22">
+        <f>E22/100</f>
+        <v/>
       </c>
       <c r="E22" t="n">
-        <v>1000</v>
+        <v>69</v>
       </c>
       <c r="F22" s="1" t="inlineStr">
         <is>
-          <t>001411</t>
+          <t>001412</t>
         </is>
       </c>
     </row>
@@ -971,18 +992,19 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>20X20X0,9MM Nest 18</t>
-        </is>
-      </c>
-      <c r="D23" t="n">
-        <v>1</v>
+          <t>20X20X0,9MM Nest 19</t>
+        </is>
+      </c>
+      <c r="D23">
+        <f>E23/100</f>
+        <v/>
       </c>
       <c r="E23" t="n">
-        <v>1000</v>
+        <v>81</v>
       </c>
       <c r="F23" s="1" t="inlineStr">
         <is>
-          <t>001412</t>
+          <t>001413</t>
         </is>
       </c>
     </row>
@@ -999,18 +1021,19 @@
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>20X20X0,9MM Nest 19</t>
-        </is>
-      </c>
-      <c r="D24" t="n">
-        <v>1</v>
+          <t>20X20X0,9MM Nest 20</t>
+        </is>
+      </c>
+      <c r="D24">
+        <f>E24/100</f>
+        <v/>
       </c>
       <c r="E24" t="n">
-        <v>1000</v>
+        <v>193</v>
       </c>
       <c r="F24" s="1" t="inlineStr">
         <is>
-          <t>001413</t>
+          <t>001414</t>
         </is>
       </c>
     </row>
@@ -1027,18 +1050,19 @@
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>20X20X0,9MM Nest 20</t>
-        </is>
-      </c>
-      <c r="D25" t="n">
-        <v>1</v>
+          <t>20X20X0,9MM Nest 21</t>
+        </is>
+      </c>
+      <c r="D25">
+        <f>E25/100</f>
+        <v/>
       </c>
       <c r="E25" t="n">
-        <v>1000</v>
+        <v>64</v>
       </c>
       <c r="F25" s="1" t="inlineStr">
         <is>
-          <t>001414</t>
+          <t>001415</t>
         </is>
       </c>
     </row>
@@ -1055,18 +1079,19 @@
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>20X20X0,9MM Nest 21</t>
-        </is>
-      </c>
-      <c r="D26" t="n">
-        <v>1</v>
+          <t>20X20X0,9MM Nest 22</t>
+        </is>
+      </c>
+      <c r="D26">
+        <f>E26/100</f>
+        <v/>
       </c>
       <c r="E26" t="n">
-        <v>1000</v>
+        <v>1</v>
       </c>
       <c r="F26" s="1" t="inlineStr">
         <is>
-          <t>001415</t>
+          <t>001416</t>
         </is>
       </c>
     </row>
@@ -1083,18 +1108,19 @@
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>20X20X0,9MM Nest 22</t>
-        </is>
-      </c>
-      <c r="D27" t="n">
-        <v>1</v>
+          <t>20X20X0,9MM Nest 23</t>
+        </is>
+      </c>
+      <c r="D27">
+        <f>E27/100</f>
+        <v/>
       </c>
       <c r="E27" t="n">
-        <v>1000</v>
+        <v>326</v>
       </c>
       <c r="F27" s="1" t="inlineStr">
         <is>
-          <t>001416</t>
+          <t>001417</t>
         </is>
       </c>
     </row>
@@ -1111,18 +1137,19 @@
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>20X20X0,9MM Nest 23</t>
-        </is>
-      </c>
-      <c r="D28" t="n">
-        <v>1</v>
+          <t>20X20X0,9MM Nest 24</t>
+        </is>
+      </c>
+      <c r="D28">
+        <f>E28/100</f>
+        <v/>
       </c>
       <c r="E28" t="n">
-        <v>1000</v>
+        <v>272</v>
       </c>
       <c r="F28" s="1" t="inlineStr">
         <is>
-          <t>001417</t>
+          <t>001418</t>
         </is>
       </c>
     </row>
@@ -1139,18 +1166,19 @@
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>20X20X0,9MM Nest 24</t>
-        </is>
-      </c>
-      <c r="D29" t="n">
-        <v>1</v>
+          <t>20X20X0,9MM Nest 25</t>
+        </is>
+      </c>
+      <c r="D29">
+        <f>E29/100</f>
+        <v/>
       </c>
       <c r="E29" t="n">
-        <v>1000</v>
+        <v>1</v>
       </c>
       <c r="F29" s="1" t="inlineStr">
         <is>
-          <t>001418</t>
+          <t>001419</t>
         </is>
       </c>
     </row>
@@ -1167,18 +1195,19 @@
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>20X20X0,9MM Nest 25</t>
-        </is>
-      </c>
-      <c r="D30" t="n">
-        <v>1</v>
+          <t>20X20X0,9MM Nest 26</t>
+        </is>
+      </c>
+      <c r="D30">
+        <f>E30/100</f>
+        <v/>
       </c>
       <c r="E30" t="n">
-        <v>1000</v>
+        <v>1</v>
       </c>
       <c r="F30" s="1" t="inlineStr">
         <is>
-          <t>001419</t>
+          <t>001420</t>
         </is>
       </c>
     </row>
@@ -1195,18 +1224,19 @@
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>20X20X0,9MM Nest 26</t>
-        </is>
-      </c>
-      <c r="D31" t="n">
-        <v>1</v>
+          <t>20X20X0,9MM Nest 27</t>
+        </is>
+      </c>
+      <c r="D31">
+        <f>E31/100</f>
+        <v/>
       </c>
       <c r="E31" t="n">
-        <v>1000</v>
+        <v>1</v>
       </c>
       <c r="F31" s="1" t="inlineStr">
         <is>
-          <t>001420</t>
+          <t>001421</t>
         </is>
       </c>
     </row>
@@ -1223,18 +1253,19 @@
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>20X20X0,9MM Nest 27</t>
-        </is>
-      </c>
-      <c r="D32" t="n">
-        <v>1</v>
+          <t>20X20X1,50MM Nest 1</t>
+        </is>
+      </c>
+      <c r="D32">
+        <f>E32/1000</f>
+        <v/>
       </c>
       <c r="E32" t="n">
-        <v>1000</v>
+        <v>331</v>
       </c>
       <c r="F32" s="1" t="inlineStr">
         <is>
-          <t>001421</t>
+          <t>001432</t>
         </is>
       </c>
     </row>
@@ -1251,18 +1282,19 @@
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>20X20X0,9MM Nest 28</t>
-        </is>
-      </c>
-      <c r="D33" t="n">
-        <v>1</v>
+          <t>20X20X1,50MM Nest 2</t>
+        </is>
+      </c>
+      <c r="D33">
+        <f>E33/1000</f>
+        <v/>
       </c>
       <c r="E33" t="n">
-        <v>1000</v>
+        <v>1</v>
       </c>
       <c r="F33" s="1" t="inlineStr">
         <is>
-          <t>001422</t>
+          <t>001433</t>
         </is>
       </c>
     </row>
@@ -1279,18 +1311,19 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>20X20X0,9MM Nest 29</t>
-        </is>
-      </c>
-      <c r="D34" t="n">
-        <v>1</v>
+          <t>20X20X1,50MM Nest 3</t>
+        </is>
+      </c>
+      <c r="D34">
+        <f>E34/1000</f>
+        <v/>
       </c>
       <c r="E34" t="n">
-        <v>1000</v>
+        <v>1</v>
       </c>
       <c r="F34" s="1" t="inlineStr">
         <is>
-          <t>001423</t>
+          <t>001434</t>
         </is>
       </c>
     </row>
@@ -1307,18 +1340,19 @@
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>20X20X0,9MM Nest 30</t>
-        </is>
-      </c>
-      <c r="D35" t="n">
-        <v>1</v>
+          <t>20X20X1,50MM Nest 4</t>
+        </is>
+      </c>
+      <c r="D35">
+        <f>E35/1000</f>
+        <v/>
       </c>
       <c r="E35" t="n">
-        <v>1000</v>
+        <v>332</v>
       </c>
       <c r="F35" s="1" t="inlineStr">
         <is>
-          <t>001424</t>
+          <t>001435</t>
         </is>
       </c>
     </row>
@@ -1335,18 +1369,19 @@
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>20X20X0,9MM Nest 31</t>
-        </is>
-      </c>
-      <c r="D36" t="n">
-        <v>1</v>
+          <t>20X20X1,50MM Nest 5</t>
+        </is>
+      </c>
+      <c r="D36">
+        <f>E36/1000</f>
+        <v/>
       </c>
       <c r="E36" t="n">
-        <v>1000</v>
+        <v>332</v>
       </c>
       <c r="F36" s="1" t="inlineStr">
         <is>
-          <t>001425</t>
+          <t>001436</t>
         </is>
       </c>
     </row>
@@ -1363,18 +1398,19 @@
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>20X20X0,9MM Nest 32</t>
-        </is>
-      </c>
-      <c r="D37" t="n">
-        <v>1</v>
+          <t>20X20X1,50MM Nest 6</t>
+        </is>
+      </c>
+      <c r="D37">
+        <f>E37/1000</f>
+        <v/>
       </c>
       <c r="E37" t="n">
-        <v>1000</v>
+        <v>332</v>
       </c>
       <c r="F37" s="1" t="inlineStr">
         <is>
-          <t>001426</t>
+          <t>001437</t>
         </is>
       </c>
     </row>
@@ -1391,18 +1427,19 @@
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>20X20X0,9MM Nest 33</t>
-        </is>
-      </c>
-      <c r="D38" t="n">
-        <v>1</v>
+          <t>20X20X1,50MM Nest 7</t>
+        </is>
+      </c>
+      <c r="D38">
+        <f>E38/1000</f>
+        <v/>
       </c>
       <c r="E38" t="n">
-        <v>1000</v>
+        <v>1</v>
       </c>
       <c r="F38" s="1" t="inlineStr">
         <is>
-          <t>001427</t>
+          <t>001438</t>
         </is>
       </c>
     </row>
@@ -1414,23 +1451,24 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>Laser Tube</t>
+          <t>Laser Chapa</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>20X20X0,9MM Nest 34</t>
-        </is>
-      </c>
-      <c r="D39" t="n">
-        <v>1</v>
+          <t>0,75 Nest 1</t>
+        </is>
+      </c>
+      <c r="D39">
+        <f>E39/1000</f>
+        <v/>
       </c>
       <c r="E39" t="n">
-        <v>1000</v>
+        <v>57</v>
       </c>
       <c r="F39" s="1" t="inlineStr">
         <is>
-          <t>001428</t>
+          <t>000311</t>
         </is>
       </c>
     </row>
@@ -1442,23 +1480,24 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>Laser Tube</t>
+          <t>Laser Chapa</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>20X20X0,9MM Nest 35</t>
-        </is>
-      </c>
-      <c r="D40" t="n">
-        <v>1</v>
+          <t>0,75 Nest 2</t>
+        </is>
+      </c>
+      <c r="D40">
+        <f>E40/1000</f>
+        <v/>
       </c>
       <c r="E40" t="n">
-        <v>1000</v>
+        <v>2</v>
       </c>
       <c r="F40" s="1" t="inlineStr">
         <is>
-          <t>001429</t>
+          <t>000312</t>
         </is>
       </c>
     </row>
@@ -1470,23 +1509,24 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>Laser Tube</t>
+          <t>Laser Chapa</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>20X20X0,9MM Nest 36</t>
-        </is>
-      </c>
-      <c r="D41" t="n">
-        <v>1</v>
+          <t>0,75 Nest 3</t>
+        </is>
+      </c>
+      <c r="D41">
+        <f>E41/1000</f>
+        <v/>
       </c>
       <c r="E41" t="n">
-        <v>1000</v>
+        <v>1</v>
       </c>
       <c r="F41" s="1" t="inlineStr">
         <is>
-          <t>001430</t>
+          <t>000313</t>
         </is>
       </c>
     </row>
@@ -1498,23 +1538,24 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>Laser Tube</t>
+          <t>Laser Chapa</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>20X20X0,9MM Nest 37</t>
-        </is>
-      </c>
-      <c r="D42" t="n">
-        <v>1</v>
+          <t>0,75 Nest 4</t>
+        </is>
+      </c>
+      <c r="D42">
+        <f>E42/1000</f>
+        <v/>
       </c>
       <c r="E42" t="n">
-        <v>1000</v>
+        <v>1</v>
       </c>
       <c r="F42" s="1" t="inlineStr">
         <is>
-          <t>001431</t>
+          <t>000314</t>
         </is>
       </c>
     </row>
@@ -1526,12 +1567,12 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>Laser Tube</t>
+          <t>Laser Chapa</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>20X20X1,50MM Nest 1</t>
+          <t>0,75 Nest 5</t>
         </is>
       </c>
       <c r="D43">
@@ -1539,11 +1580,11 @@
         <v/>
       </c>
       <c r="E43" t="n">
-        <v>331</v>
+        <v>1</v>
       </c>
       <c r="F43" s="1" t="inlineStr">
         <is>
-          <t>001432</t>
+          <t>000315</t>
         </is>
       </c>
     </row>
@@ -1555,12 +1596,12 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>Laser Tube</t>
+          <t>Laser Chapa</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>20X20X1,50MM Nest 2</t>
+          <t>0,75 Nest 6</t>
         </is>
       </c>
       <c r="D44">
@@ -1568,11 +1609,11 @@
         <v/>
       </c>
       <c r="E44" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="F44" s="1" t="inlineStr">
         <is>
-          <t>001433</t>
+          <t>000316</t>
         </is>
       </c>
     </row>
@@ -1584,12 +1625,12 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>Laser Tube</t>
+          <t>Laser Chapa</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>20X20X1,50MM Nest 3</t>
+          <t>0,75 Nest 7</t>
         </is>
       </c>
       <c r="D45">
@@ -1597,11 +1638,11 @@
         <v/>
       </c>
       <c r="E45" t="n">
-        <v>1</v>
+        <v>11</v>
       </c>
       <c r="F45" s="1" t="inlineStr">
         <is>
-          <t>001434</t>
+          <t>000317</t>
         </is>
       </c>
     </row>
@@ -1613,12 +1654,12 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>Laser Tube</t>
+          <t>Laser Chapa</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>20X20X1,50MM Nest 4</t>
+          <t>0,75 Nest 8</t>
         </is>
       </c>
       <c r="D46">
@@ -1626,11 +1667,11 @@
         <v/>
       </c>
       <c r="E46" t="n">
-        <v>332</v>
+        <v>1</v>
       </c>
       <c r="F46" s="1" t="inlineStr">
         <is>
-          <t>001435</t>
+          <t>000318</t>
         </is>
       </c>
     </row>
@@ -1642,12 +1683,12 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>Laser Tube</t>
+          <t>Laser Chapa</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>20X20X1,50MM Nest 5</t>
+          <t>0,75 Nest 9</t>
         </is>
       </c>
       <c r="D47">
@@ -1655,11 +1696,11 @@
         <v/>
       </c>
       <c r="E47" t="n">
-        <v>332</v>
+        <v>5</v>
       </c>
       <c r="F47" s="1" t="inlineStr">
         <is>
-          <t>001436</t>
+          <t>000319</t>
         </is>
       </c>
     </row>
@@ -1671,12 +1712,12 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>Laser Tube</t>
+          <t>Laser Chapa</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>20X20X1,50MM Nest 6</t>
+          <t>0,75 Nest 10</t>
         </is>
       </c>
       <c r="D48">
@@ -1684,11 +1725,11 @@
         <v/>
       </c>
       <c r="E48" t="n">
-        <v>332</v>
+        <v>1</v>
       </c>
       <c r="F48" s="1" t="inlineStr">
         <is>
-          <t>001437</t>
+          <t>001449</t>
         </is>
       </c>
     </row>
@@ -1700,12 +1741,12 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>Laser Tube</t>
+          <t>Laser Chapa</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>20X20X1,50MM Nest 7</t>
+          <t>0,75 Nest 11</t>
         </is>
       </c>
       <c r="D49">
@@ -1717,7 +1758,7 @@
       </c>
       <c r="F49" s="1" t="inlineStr">
         <is>
-          <t>001438</t>
+          <t>001450</t>
         </is>
       </c>
     </row>
@@ -1734,19 +1775,19 @@
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>0,75 Nest 1</t>
+          <t>0,75 Nest 12</t>
         </is>
       </c>
       <c r="D50">
-        <f>E50/1700</f>
+        <f>E50/1000</f>
         <v/>
       </c>
       <c r="E50" t="n">
-        <v>24</v>
+        <v>79</v>
       </c>
       <c r="F50" s="1" t="inlineStr">
         <is>
-          <t>000311</t>
+          <t>001451</t>
         </is>
       </c>
     </row>
@@ -1763,19 +1804,19 @@
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>0,75 Nest 2</t>
+          <t>0,75 Nest 13</t>
         </is>
       </c>
       <c r="D51">
-        <f>E51/1700</f>
+        <f>E51/1000</f>
         <v/>
       </c>
       <c r="E51" t="n">
-        <v>28</v>
+        <v>247</v>
       </c>
       <c r="F51" s="1" t="inlineStr">
         <is>
-          <t>000312</t>
+          <t>001452</t>
         </is>
       </c>
     </row>
@@ -1792,19 +1833,19 @@
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>0,75 Nest 3</t>
+          <t>0,75 Nest 14</t>
         </is>
       </c>
       <c r="D52">
-        <f>E52/1700</f>
+        <f>E52/1000</f>
         <v/>
       </c>
       <c r="E52" t="n">
-        <v>35</v>
+        <v>2</v>
       </c>
       <c r="F52" s="1" t="inlineStr">
         <is>
-          <t>000313</t>
+          <t>001453</t>
         </is>
       </c>
     </row>
@@ -1821,19 +1862,19 @@
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>0,75 Nest 4</t>
+          <t>0,75 Nest 15</t>
         </is>
       </c>
       <c r="D53">
-        <f>E53/1700</f>
+        <f>E53/1000</f>
         <v/>
       </c>
       <c r="E53" t="n">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="F53" s="1" t="inlineStr">
         <is>
-          <t>000314</t>
+          <t>001454</t>
         </is>
       </c>
     </row>
@@ -1850,11 +1891,11 @@
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>0,75 Nest 5</t>
+          <t>0,75 Nest 16</t>
         </is>
       </c>
       <c r="D54">
-        <f>E54/1700</f>
+        <f>E54/1000</f>
         <v/>
       </c>
       <c r="E54" t="n">
@@ -1862,7 +1903,7 @@
       </c>
       <c r="F54" s="1" t="inlineStr">
         <is>
-          <t>000315</t>
+          <t>001455</t>
         </is>
       </c>
     </row>
@@ -1879,11 +1920,11 @@
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>0,75 Nest 6</t>
+          <t>0,75 Nest 17</t>
         </is>
       </c>
       <c r="D55">
-        <f>E55/1700</f>
+        <f>E55/1000</f>
         <v/>
       </c>
       <c r="E55" t="n">
@@ -1891,7 +1932,7 @@
       </c>
       <c r="F55" s="1" t="inlineStr">
         <is>
-          <t>000316</t>
+          <t>001456</t>
         </is>
       </c>
     </row>
@@ -1908,19 +1949,19 @@
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>0,75 Nest 7</t>
+          <t>0,9 Nest 1</t>
         </is>
       </c>
       <c r="D56">
-        <f>E56/1700</f>
+        <f>E56/1000</f>
         <v/>
       </c>
       <c r="E56" t="n">
-        <v>424</v>
+        <v>869</v>
       </c>
       <c r="F56" s="1" t="inlineStr">
         <is>
-          <t>000317</t>
+          <t>000320</t>
         </is>
       </c>
     </row>
@@ -1937,19 +1978,19 @@
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>0,75 Nest 8</t>
+          <t>0,9 Nest 2</t>
         </is>
       </c>
       <c r="D57">
-        <f>E57/1700</f>
+        <f>E57/1000</f>
         <v/>
       </c>
       <c r="E57" t="n">
-        <v>63</v>
+        <v>84</v>
       </c>
       <c r="F57" s="1" t="inlineStr">
         <is>
-          <t>000318</t>
+          <t>000321</t>
         </is>
       </c>
     </row>
@@ -1966,19 +2007,19 @@
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>0,75 Nest 9</t>
+          <t>0,9 Nest 3</t>
         </is>
       </c>
       <c r="D58">
-        <f>E58/1700</f>
+        <f>E58/1000</f>
         <v/>
       </c>
       <c r="E58" t="n">
-        <v>1</v>
+        <v>217</v>
       </c>
       <c r="F58" s="1" t="inlineStr">
         <is>
-          <t>000319</t>
+          <t>000322</t>
         </is>
       </c>
     </row>
@@ -1995,19 +2036,19 @@
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>0,9 Nest 1</t>
+          <t>0,9 Nest 4</t>
         </is>
       </c>
       <c r="D59">
-        <f>E59/1700</f>
+        <f>E59/1000</f>
         <v/>
       </c>
       <c r="E59" t="n">
-        <v>196</v>
+        <v>119</v>
       </c>
       <c r="F59" s="1" t="inlineStr">
         <is>
-          <t>000320</t>
+          <t>000323</t>
         </is>
       </c>
     </row>
@@ -2024,11 +2065,11 @@
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>0,9 Nest 2</t>
+          <t>0,9 Nest 5</t>
         </is>
       </c>
       <c r="D60">
-        <f>E60/1700</f>
+        <f>E60/1000</f>
         <v/>
       </c>
       <c r="E60" t="n">
@@ -2036,7 +2077,7 @@
       </c>
       <c r="F60" s="1" t="inlineStr">
         <is>
-          <t>000321</t>
+          <t>000324</t>
         </is>
       </c>
     </row>
@@ -2053,19 +2094,19 @@
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>0,9 Nest 3</t>
+          <t>0,9 Nest 6</t>
         </is>
       </c>
       <c r="D61">
-        <f>E61/1700</f>
+        <f>E61/1000</f>
         <v/>
       </c>
       <c r="E61" t="n">
-        <v>43</v>
+        <v>1</v>
       </c>
       <c r="F61" s="1" t="inlineStr">
         <is>
-          <t>000322</t>
+          <t>000325</t>
         </is>
       </c>
     </row>
@@ -2082,7 +2123,7 @@
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>0,9 Nest 4</t>
+          <t>1,2 Nest 1</t>
         </is>
       </c>
       <c r="D62">
@@ -2090,11 +2131,11 @@
         <v/>
       </c>
       <c r="E62" t="n">
-        <v>2</v>
+        <v>11</v>
       </c>
       <c r="F62" s="1" t="inlineStr">
         <is>
-          <t>000323</t>
+          <t>000335</t>
         </is>
       </c>
     </row>
@@ -2111,7 +2152,7 @@
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>0,9 Nest 5</t>
+          <t>1,2 Nest 2</t>
         </is>
       </c>
       <c r="D63">
@@ -2119,11 +2160,11 @@
         <v/>
       </c>
       <c r="E63" t="n">
-        <v>12</v>
+        <v>1</v>
       </c>
       <c r="F63" s="1" t="inlineStr">
         <is>
-          <t>000324</t>
+          <t>000336</t>
         </is>
       </c>
     </row>
@@ -2140,19 +2181,19 @@
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>0,9 Nest 6</t>
+          <t>2,65 Nest 1</t>
         </is>
       </c>
       <c r="D64">
-        <f>E64/1700</f>
+        <f>E64/1000</f>
         <v/>
       </c>
       <c r="E64" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F64" s="1" t="inlineStr">
         <is>
-          <t>000325</t>
+          <t>000337</t>
         </is>
       </c>
     </row>
@@ -2169,19 +2210,19 @@
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>0,9 Nest 7</t>
+          <t>2,65 Nest 2</t>
         </is>
       </c>
       <c r="D65">
-        <f>E65/1700</f>
+        <f>E65/1000</f>
         <v/>
       </c>
       <c r="E65" t="n">
-        <v>1</v>
+        <v>99</v>
       </c>
       <c r="F65" s="1" t="inlineStr">
         <is>
-          <t>000326</t>
+          <t>000338</t>
         </is>
       </c>
     </row>
@@ -2198,19 +2239,19 @@
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>0,9 Nest 8</t>
+          <t>2,65 Nest 3</t>
         </is>
       </c>
       <c r="D66">
-        <f>E66/1700</f>
+        <f>E66/1000</f>
         <v/>
       </c>
       <c r="E66" t="n">
-        <v>100</v>
+        <v>2</v>
       </c>
       <c r="F66" s="1" t="inlineStr">
         <is>
-          <t>000327</t>
+          <t>000339</t>
         </is>
       </c>
     </row>
@@ -2227,19 +2268,19 @@
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>0,9 Nest 9</t>
+          <t>2,65 Nest 4</t>
         </is>
       </c>
       <c r="D67">
-        <f>E67/1700</f>
+        <f>E67/1000</f>
         <v/>
       </c>
       <c r="E67" t="n">
-        <v>409</v>
+        <v>219</v>
       </c>
       <c r="F67" s="1" t="inlineStr">
         <is>
-          <t>000328</t>
+          <t>000340</t>
         </is>
       </c>
     </row>
@@ -2256,19 +2297,19 @@
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>0,9 Nest 10</t>
+          <t>2,65 Nest 5</t>
         </is>
       </c>
       <c r="D68">
-        <f>E68/1700</f>
+        <f>E68/1000</f>
         <v/>
       </c>
       <c r="E68" t="n">
-        <v>1114</v>
+        <v>1</v>
       </c>
       <c r="F68" s="1" t="inlineStr">
         <is>
-          <t>000329</t>
+          <t>000341</t>
         </is>
       </c>
     </row>
@@ -2285,19 +2326,19 @@
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>0,9 Nest 11</t>
+          <t>2,65 Nest 6</t>
         </is>
       </c>
       <c r="D69">
-        <f>E69/1700</f>
+        <f>E69/1000</f>
         <v/>
       </c>
       <c r="E69" t="n">
-        <v>355</v>
+        <v>1</v>
       </c>
       <c r="F69" s="1" t="inlineStr">
         <is>
-          <t>000330</t>
+          <t>000342</t>
         </is>
       </c>
     </row>
@@ -2314,19 +2355,19 @@
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>0,9 Nest 12</t>
+          <t>2,65 Nest 7</t>
         </is>
       </c>
       <c r="D70">
-        <f>E70/1700</f>
+        <f>E70/1000</f>
         <v/>
       </c>
       <c r="E70" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="F70" s="1" t="inlineStr">
         <is>
-          <t>000331</t>
+          <t>000343</t>
         </is>
       </c>
     </row>
@@ -2343,11 +2384,11 @@
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>0,9 Nest 13</t>
+          <t>2,65 Nest 8</t>
         </is>
       </c>
       <c r="D71">
-        <f>E71/1700</f>
+        <f>E71/1000</f>
         <v/>
       </c>
       <c r="E71" t="n">
@@ -2355,7 +2396,7 @@
       </c>
       <c r="F71" s="1" t="inlineStr">
         <is>
-          <t>000332</t>
+          <t>000344</t>
         </is>
       </c>
     </row>
@@ -2367,24 +2408,23 @@
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>Laser Chapa</t>
+          <t>Serra</t>
         </is>
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>0,9 Nest 14</t>
-        </is>
-      </c>
-      <c r="D72">
-        <f>E72/1700</f>
-        <v/>
+          <t>Tubo Bdj 433 MM</t>
+        </is>
+      </c>
+      <c r="D72" t="n">
+        <v>5</v>
       </c>
       <c r="E72" t="n">
-        <v>1</v>
+        <v>5000</v>
       </c>
       <c r="F72" s="1" t="inlineStr">
         <is>
-          <t>000333</t>
+          <t>000379</t>
         </is>
       </c>
     </row>
@@ -2396,24 +2436,23 @@
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>Laser Chapa</t>
+          <t>Serra</t>
         </is>
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>0,9 Nest 15</t>
-        </is>
-      </c>
-      <c r="D73">
-        <f>E73/1700</f>
-        <v/>
+          <t>Tubo Bdj 493 MM</t>
+        </is>
+      </c>
+      <c r="D73" t="n">
+        <v>5</v>
       </c>
       <c r="E73" t="n">
-        <v>1</v>
+        <v>5000</v>
       </c>
       <c r="F73" s="1" t="inlineStr">
         <is>
-          <t>000334</t>
+          <t>000380</t>
         </is>
       </c>
     </row>
@@ -2425,24 +2464,23 @@
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>Laser Chapa</t>
+          <t>Dobradeira de Arames</t>
         </is>
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>1,2 Nest 1</t>
-        </is>
-      </c>
-      <c r="D74">
-        <f>E74/1700</f>
-        <v/>
+          <t>Arame Toldo Lateral</t>
+        </is>
+      </c>
+      <c r="D74" t="n">
+        <v>2</v>
       </c>
       <c r="E74" t="n">
-        <v>11</v>
+        <v>2000</v>
       </c>
       <c r="F74" s="1" t="inlineStr">
         <is>
-          <t>000335</t>
+          <t>001439</t>
         </is>
       </c>
     </row>
@@ -2454,24 +2492,23 @@
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>Laser Chapa</t>
+          <t>Dobradeira de Arames</t>
         </is>
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>1,2 Nest 2</t>
-        </is>
-      </c>
-      <c r="D75">
-        <f>E75/1700</f>
-        <v/>
+          <t>Arame Toldo Trecho Reto</t>
+        </is>
+      </c>
+      <c r="D75" t="n">
+        <v>3</v>
       </c>
       <c r="E75" t="n">
-        <v>1</v>
+        <v>3000</v>
       </c>
       <c r="F75" s="1" t="inlineStr">
         <is>
-          <t>000336</t>
+          <t>001440</t>
         </is>
       </c>
     </row>
@@ -2483,24 +2520,23 @@
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>Laser Chapa</t>
+          <t>Dobradeira de Chapas</t>
         </is>
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>2,65 Nest 1</t>
-        </is>
-      </c>
-      <c r="D76">
-        <f>E76/1000</f>
-        <v/>
+          <t>J 1732 mm</t>
+        </is>
+      </c>
+      <c r="D76" t="n">
+        <v>4</v>
       </c>
       <c r="E76" t="n">
-        <v>1</v>
+        <v>4000</v>
       </c>
       <c r="F76" s="1" t="inlineStr">
         <is>
-          <t>000337</t>
+          <t>000346</t>
         </is>
       </c>
     </row>
@@ -2512,24 +2548,23 @@
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>Laser Chapa</t>
+          <t>Dobradeira de Chapas</t>
         </is>
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>2,65 Nest 2</t>
-        </is>
-      </c>
-      <c r="D77">
-        <f>E77/1000</f>
-        <v/>
+          <t>J 333 mm</t>
+        </is>
+      </c>
+      <c r="D77" t="n">
+        <v>2</v>
       </c>
       <c r="E77" t="n">
-        <v>99</v>
+        <v>2000</v>
       </c>
       <c r="F77" s="1" t="inlineStr">
         <is>
-          <t>000338</t>
+          <t>000347</t>
         </is>
       </c>
     </row>
@@ -2541,24 +2576,23 @@
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>Laser Chapa</t>
+          <t>Dobradeira de Chapas</t>
         </is>
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>2,65 Nest 3</t>
-        </is>
-      </c>
-      <c r="D78">
-        <f>E78/1000</f>
-        <v/>
+          <t>J 1028 mm</t>
+        </is>
+      </c>
+      <c r="D78" t="n">
+        <v>1</v>
       </c>
       <c r="E78" t="n">
-        <v>2</v>
+        <v>1000</v>
       </c>
       <c r="F78" s="1" t="inlineStr">
         <is>
-          <t>000339</t>
+          <t>000348</t>
         </is>
       </c>
     </row>
@@ -2570,24 +2604,23 @@
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>Laser Chapa</t>
+          <t>Dobradeira de Chapas</t>
         </is>
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>2,65 Nest 4</t>
-        </is>
-      </c>
-      <c r="D79">
-        <f>E79/1000</f>
-        <v/>
+          <t>Fechamento Saia</t>
+        </is>
+      </c>
+      <c r="D79" t="n">
+        <v>1</v>
       </c>
       <c r="E79" t="n">
-        <v>219</v>
+        <v>1000</v>
       </c>
       <c r="F79" s="1" t="inlineStr">
         <is>
-          <t>000340</t>
+          <t>000349</t>
         </is>
       </c>
     </row>
@@ -2599,24 +2632,23 @@
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>Laser Chapa</t>
+          <t>Dobradeira de Chapas</t>
         </is>
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>2,65 Nest 5</t>
-        </is>
-      </c>
-      <c r="D80">
-        <f>E80/1000</f>
-        <v/>
+          <t>Fechamento Parachoque Móvel</t>
+        </is>
+      </c>
+      <c r="D80" t="n">
+        <v>1</v>
       </c>
       <c r="E80" t="n">
-        <v>1</v>
+        <v>1000</v>
       </c>
       <c r="F80" s="1" t="inlineStr">
         <is>
-          <t>000341</t>
+          <t>000350</t>
         </is>
       </c>
     </row>
@@ -2628,24 +2660,23 @@
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>Laser Chapa</t>
+          <t>Dobradeira de Chapas</t>
         </is>
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>2,65 Nest 6</t>
-        </is>
-      </c>
-      <c r="D81">
-        <f>E81/1000</f>
-        <v/>
+          <t>Chapa Frontal Testeira</t>
+        </is>
+      </c>
+      <c r="D81" t="n">
+        <v>1</v>
       </c>
       <c r="E81" t="n">
-        <v>1</v>
+        <v>1000</v>
       </c>
       <c r="F81" s="1" t="inlineStr">
         <is>
-          <t>000342</t>
+          <t>000351</t>
         </is>
       </c>
     </row>
@@ -2657,24 +2688,23 @@
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>Laser Chapa</t>
+          <t>Dobradeira de Chapas</t>
         </is>
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>2,65 Nest 7</t>
-        </is>
-      </c>
-      <c r="D82">
-        <f>E82/1000</f>
-        <v/>
+          <t>Chapa Central Fixação Toldo</t>
+        </is>
+      </c>
+      <c r="D82" t="n">
+        <v>1</v>
       </c>
       <c r="E82" t="n">
-        <v>5</v>
+        <v>1000</v>
       </c>
       <c r="F82" s="1" t="inlineStr">
         <is>
-          <t>000343</t>
+          <t>000352</t>
         </is>
       </c>
     </row>
@@ -2686,24 +2716,23 @@
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>Laser Chapa</t>
+          <t>Dobradeira de Chapas</t>
         </is>
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>2,65 Nest 8</t>
-        </is>
-      </c>
-      <c r="D83">
-        <f>E83/1000</f>
-        <v/>
+          <t>Encaixe Parachoque Direito</t>
+        </is>
+      </c>
+      <c r="D83" t="n">
+        <v>3</v>
       </c>
       <c r="E83" t="n">
-        <v>1</v>
+        <v>3000</v>
       </c>
       <c r="F83" s="1" t="inlineStr">
         <is>
-          <t>000344</t>
+          <t>000353</t>
         </is>
       </c>
     </row>
@@ -2715,23 +2744,23 @@
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>Serra</t>
+          <t>Dobradeira de Chapas</t>
         </is>
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>Tubo Bdj 433 MM</t>
+          <t>Encaixe Parachoque Esquerda</t>
         </is>
       </c>
       <c r="D84" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="E84" t="n">
-        <v>5000</v>
+        <v>2000</v>
       </c>
       <c r="F84" s="1" t="inlineStr">
         <is>
-          <t>000379</t>
+          <t>000354</t>
         </is>
       </c>
     </row>
@@ -2743,23 +2772,23 @@
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>Serra</t>
+          <t>Dobradeira de Chapas</t>
         </is>
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>Tubo Bdj 493 MM</t>
+          <t>Bdj Esquerda Amassamento</t>
         </is>
       </c>
       <c r="D85" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="E85" t="n">
-        <v>5000</v>
+        <v>4000</v>
       </c>
       <c r="F85" s="1" t="inlineStr">
         <is>
-          <t>000380</t>
+          <t>000355</t>
         </is>
       </c>
     </row>
@@ -2771,23 +2800,23 @@
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>Dobradeira de Arames</t>
+          <t>Dobradeira de Chapas</t>
         </is>
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>Arame Toldo Lateral</t>
+          <t>Bdj Esquerda Dobra</t>
         </is>
       </c>
       <c r="D86" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="E86" t="n">
-        <v>2000</v>
+        <v>4000</v>
       </c>
       <c r="F86" s="1" t="inlineStr">
         <is>
-          <t>001439</t>
+          <t>000356</t>
         </is>
       </c>
     </row>
@@ -2799,23 +2828,23 @@
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>Dobradeira de Arames</t>
+          <t>Dobradeira de Chapas</t>
         </is>
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>Arame Toldo Trecho Reto</t>
+          <t>Bdj Direita Amassamento</t>
         </is>
       </c>
       <c r="D87" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E87" t="n">
-        <v>3000</v>
+        <v>4000</v>
       </c>
       <c r="F87" s="1" t="inlineStr">
         <is>
-          <t>001440</t>
+          <t>000357</t>
         </is>
       </c>
     </row>
@@ -2832,7 +2861,7 @@
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>J 1732 mm</t>
+          <t>Bdj Direita Dobra</t>
         </is>
       </c>
       <c r="D88" t="n">
@@ -2843,7 +2872,7 @@
       </c>
       <c r="F88" s="1" t="inlineStr">
         <is>
-          <t>000346</t>
+          <t>000358</t>
         </is>
       </c>
     </row>
@@ -2860,18 +2889,18 @@
       </c>
       <c r="C89" t="inlineStr">
         <is>
-          <t>J 333 mm</t>
+          <t>Bdj Esquerda Base Amassamento</t>
         </is>
       </c>
       <c r="D89" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E89" t="n">
-        <v>2000</v>
+        <v>1000</v>
       </c>
       <c r="F89" s="1" t="inlineStr">
         <is>
-          <t>000347</t>
+          <t>000359</t>
         </is>
       </c>
     </row>
@@ -2888,7 +2917,7 @@
       </c>
       <c r="C90" t="inlineStr">
         <is>
-          <t>J 1028 mm</t>
+          <t>Bdj Esquerda Base Dobra</t>
         </is>
       </c>
       <c r="D90" t="n">
@@ -2899,7 +2928,7 @@
       </c>
       <c r="F90" s="1" t="inlineStr">
         <is>
-          <t>000348</t>
+          <t>000360</t>
         </is>
       </c>
     </row>
@@ -2916,7 +2945,7 @@
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>Fechamento Saia</t>
+          <t>Bdj Direita Base Amassamento</t>
         </is>
       </c>
       <c r="D91" t="n">
@@ -2927,7 +2956,7 @@
       </c>
       <c r="F91" s="1" t="inlineStr">
         <is>
-          <t>000349</t>
+          <t>000361</t>
         </is>
       </c>
     </row>
@@ -2944,7 +2973,7 @@
       </c>
       <c r="C92" t="inlineStr">
         <is>
-          <t>Fechamento Parachoque Móvel</t>
+          <t>Bdj Direita Base Dobra</t>
         </is>
       </c>
       <c r="D92" t="n">
@@ -2955,7 +2984,7 @@
       </c>
       <c r="F92" s="1" t="inlineStr">
         <is>
-          <t>000350</t>
+          <t>000362</t>
         </is>
       </c>
     </row>
@@ -2972,18 +3001,18 @@
       </c>
       <c r="C93" t="inlineStr">
         <is>
-          <t>Chapa Frontal Testeira</t>
+          <t>Chapa Gancho Pallet</t>
         </is>
       </c>
       <c r="D93" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E93" t="n">
         <v>1000</v>
       </c>
       <c r="F93" s="1" t="inlineStr">
         <is>
-          <t>000351</t>
+          <t>000363</t>
         </is>
       </c>
     </row>
@@ -2995,12 +3024,12 @@
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>Dobradeira de Chapas</t>
+          <t>Solda Mig</t>
         </is>
       </c>
       <c r="C94" t="inlineStr">
         <is>
-          <t>Chapa Central Fixação Toldo</t>
+          <t>Lateral Esquerda Tubular</t>
         </is>
       </c>
       <c r="D94" t="n">
@@ -3011,7 +3040,7 @@
       </c>
       <c r="F94" s="1" t="inlineStr">
         <is>
-          <t>000352</t>
+          <t>000364</t>
         </is>
       </c>
     </row>
@@ -3023,23 +3052,23 @@
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>Dobradeira de Chapas</t>
+          <t>Solda Mig</t>
         </is>
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>Encaixe Parachoque Direito</t>
+          <t>Lateral Direita Tubular</t>
         </is>
       </c>
       <c r="D95" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="E95" t="n">
-        <v>3000</v>
+        <v>1000</v>
       </c>
       <c r="F95" s="1" t="inlineStr">
         <is>
-          <t>000353</t>
+          <t>000365</t>
         </is>
       </c>
     </row>
@@ -3051,23 +3080,23 @@
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>Dobradeira de Chapas</t>
+          <t>Solda Mig</t>
         </is>
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t>Encaixe Parachoque Esquerda</t>
+          <t>Lateral Esquerda Chaparia + Triângulo 2,65</t>
         </is>
       </c>
       <c r="D96" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E96" t="n">
-        <v>2000</v>
+        <v>1000</v>
       </c>
       <c r="F96" s="1" t="inlineStr">
         <is>
-          <t>000354</t>
+          <t>000366</t>
         </is>
       </c>
     </row>
@@ -3079,23 +3108,23 @@
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>Dobradeira de Chapas</t>
+          <t>Solda Mig</t>
         </is>
       </c>
       <c r="C97" t="inlineStr">
         <is>
-          <t>Bdj Esquerda Amassamento</t>
+          <t>Lateral Direita Chaparia + Triângulo 2,65</t>
         </is>
       </c>
       <c r="D97" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="E97" t="n">
-        <v>4000</v>
+        <v>1000</v>
       </c>
       <c r="F97" s="1" t="inlineStr">
         <is>
-          <t>000355</t>
+          <t>000367</t>
         </is>
       </c>
     </row>
@@ -3107,23 +3136,23 @@
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>Dobradeira de Chapas</t>
+          <t>Solda Mig</t>
         </is>
       </c>
       <c r="C98" t="inlineStr">
         <is>
-          <t>Bdj Esquerda Dobra</t>
+          <t>Lateral Esquerda Arruela Quadrada 2,65</t>
         </is>
       </c>
       <c r="D98" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="E98" t="n">
-        <v>4000</v>
+        <v>1000</v>
       </c>
       <c r="F98" s="1" t="inlineStr">
         <is>
-          <t>000356</t>
+          <t>000368</t>
         </is>
       </c>
     </row>
@@ -3135,23 +3164,23 @@
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>Dobradeira de Chapas</t>
+          <t>Solda Mig</t>
         </is>
       </c>
       <c r="C99" t="inlineStr">
         <is>
-          <t>Bdj Direita Amassamento</t>
+          <t>Lateral Direita Arruela Quadrada 2,65</t>
         </is>
       </c>
       <c r="D99" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="E99" t="n">
-        <v>4000</v>
+        <v>1000</v>
       </c>
       <c r="F99" s="1" t="inlineStr">
         <is>
-          <t>000357</t>
+          <t>000369</t>
         </is>
       </c>
     </row>
@@ -3163,23 +3192,23 @@
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>Dobradeira de Chapas</t>
+          <t>Solda Mig</t>
         </is>
       </c>
       <c r="C100" t="inlineStr">
         <is>
-          <t>Bdj Direita Dobra</t>
+          <t>Quadro Cremalheira</t>
         </is>
       </c>
       <c r="D100" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="E100" t="n">
-        <v>4000</v>
+        <v>1000</v>
       </c>
       <c r="F100" s="1" t="inlineStr">
         <is>
-          <t>000358</t>
+          <t>000386</t>
         </is>
       </c>
     </row>
@@ -3191,12 +3220,12 @@
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t>Dobradeira de Chapas</t>
+          <t>Solda Mig</t>
         </is>
       </c>
       <c r="C101" t="inlineStr">
         <is>
-          <t>Bdj Esquerda Base Amassamento</t>
+          <t>Levantamento Corpo</t>
         </is>
       </c>
       <c r="D101" t="n">
@@ -3207,7 +3236,7 @@
       </c>
       <c r="F101" s="1" t="inlineStr">
         <is>
-          <t>000359</t>
+          <t>000370</t>
         </is>
       </c>
     </row>
@@ -3219,12 +3248,12 @@
       </c>
       <c r="B102" t="inlineStr">
         <is>
-          <t>Dobradeira de Chapas</t>
+          <t>Solda Mig</t>
         </is>
       </c>
       <c r="C102" t="inlineStr">
         <is>
-          <t>Bdj Esquerda Base Dobra</t>
+          <t>Chaparia Testeira + Saia + Canaletas</t>
         </is>
       </c>
       <c r="D102" t="n">
@@ -3235,7 +3264,7 @@
       </c>
       <c r="F102" s="1" t="inlineStr">
         <is>
-          <t>000360</t>
+          <t>000371</t>
         </is>
       </c>
     </row>
@@ -3247,23 +3276,23 @@
       </c>
       <c r="B103" t="inlineStr">
         <is>
-          <t>Dobradeira de Chapas</t>
+          <t>Solda Mig</t>
         </is>
       </c>
       <c r="C103" t="inlineStr">
         <is>
-          <t>Bdj Direita Base Amassamento</t>
+          <t>Bdj Esquerda Tubo + Mão francesa (inferior)</t>
         </is>
       </c>
       <c r="D103" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="E103" t="n">
-        <v>1000</v>
+        <v>4000</v>
       </c>
       <c r="F103" s="1" t="inlineStr">
         <is>
-          <t>000361</t>
+          <t>001441</t>
         </is>
       </c>
     </row>
@@ -3275,23 +3304,23 @@
       </c>
       <c r="B104" t="inlineStr">
         <is>
-          <t>Dobradeira de Chapas</t>
+          <t>Solda Mig</t>
         </is>
       </c>
       <c r="C104" t="inlineStr">
         <is>
-          <t>Bdj Direita Base Dobra</t>
+          <t>Bdj Direita Tubo + Mão francesa (inferior)</t>
         </is>
       </c>
       <c r="D104" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="E104" t="n">
-        <v>1000</v>
+        <v>4000</v>
       </c>
       <c r="F104" s="1" t="inlineStr">
         <is>
-          <t>000362</t>
+          <t>001442</t>
         </is>
       </c>
     </row>
@@ -3303,23 +3332,23 @@
       </c>
       <c r="B105" t="inlineStr">
         <is>
-          <t>Dobradeira de Chapas</t>
+          <t>Solda Mig</t>
         </is>
       </c>
       <c r="C105" t="inlineStr">
         <is>
-          <t>Chapa Gancho Pallet</t>
+          <t>Bdj Esquerda Base Tubo + Mão francesa (inferior)</t>
         </is>
       </c>
       <c r="D105" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E105" t="n">
         <v>1000</v>
       </c>
       <c r="F105" s="1" t="inlineStr">
         <is>
-          <t>000363</t>
+          <t>001443</t>
         </is>
       </c>
     </row>
@@ -3336,7 +3365,7 @@
       </c>
       <c r="C106" t="inlineStr">
         <is>
-          <t>Lateral Esquerda Tubular</t>
+          <t>Bdj Direita Base Tubo + Mão francesa (inferior)</t>
         </is>
       </c>
       <c r="D106" t="n">
@@ -3347,7 +3376,7 @@
       </c>
       <c r="F106" s="1" t="inlineStr">
         <is>
-          <t>000364</t>
+          <t>001444</t>
         </is>
       </c>
     </row>
@@ -3364,18 +3393,18 @@
       </c>
       <c r="C107" t="inlineStr">
         <is>
-          <t>Lateral Direita Tubular</t>
+          <t>Bdj Esquerda Tubo + Mão francesa (superior)</t>
         </is>
       </c>
       <c r="D107" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="E107" t="n">
-        <v>1000</v>
+        <v>4000</v>
       </c>
       <c r="F107" s="1" t="inlineStr">
         <is>
-          <t>000365</t>
+          <t>001445</t>
         </is>
       </c>
     </row>
@@ -3392,18 +3421,18 @@
       </c>
       <c r="C108" t="inlineStr">
         <is>
-          <t>Lateral Esquerda Chaparia + Triângulo 2,65</t>
+          <t>Bdj Direita Tubo + Mão francesa (superior)</t>
         </is>
       </c>
       <c r="D108" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="E108" t="n">
-        <v>1000</v>
+        <v>4000</v>
       </c>
       <c r="F108" s="1" t="inlineStr">
         <is>
-          <t>000366</t>
+          <t>001446</t>
         </is>
       </c>
     </row>
@@ -3420,7 +3449,7 @@
       </c>
       <c r="C109" t="inlineStr">
         <is>
-          <t>Lateral Direita Chaparia + Triângulo 2,65</t>
+          <t>Bdj Esquerda Base Tubo + Mão francesa (superior)</t>
         </is>
       </c>
       <c r="D109" t="n">
@@ -3431,7 +3460,7 @@
       </c>
       <c r="F109" s="1" t="inlineStr">
         <is>
-          <t>000367</t>
+          <t>001447</t>
         </is>
       </c>
     </row>
@@ -3448,7 +3477,7 @@
       </c>
       <c r="C110" t="inlineStr">
         <is>
-          <t>Lateral Esquerda Arruela Quadrada 2,65</t>
+          <t>Bdj Direita Base Tubo + Mão francesa (superior)</t>
         </is>
       </c>
       <c r="D110" t="n">
@@ -3459,7 +3488,7 @@
       </c>
       <c r="F110" s="1" t="inlineStr">
         <is>
-          <t>000368</t>
+          <t>001448</t>
         </is>
       </c>
     </row>
@@ -3476,7 +3505,7 @@
       </c>
       <c r="C111" t="inlineStr">
         <is>
-          <t>Lateral Direita Arruela Quadrada 2,65</t>
+          <t>Aramado Toldo</t>
         </is>
       </c>
       <c r="D111" t="n">
@@ -3487,7 +3516,7 @@
       </c>
       <c r="F111" s="1" t="inlineStr">
         <is>
-          <t>000369</t>
+          <t>000376</t>
         </is>
       </c>
     </row>
@@ -3504,7 +3533,7 @@
       </c>
       <c r="C112" t="inlineStr">
         <is>
-          <t>Quadro Cremalheira</t>
+          <t>Aramado Toldo + Chapa Fixação</t>
         </is>
       </c>
       <c r="D112" t="n">
@@ -3515,7 +3544,7 @@
       </c>
       <c r="F112" s="1" t="inlineStr">
         <is>
-          <t>000386</t>
+          <t>000377</t>
         </is>
       </c>
     </row>
@@ -3532,7 +3561,7 @@
       </c>
       <c r="C113" t="inlineStr">
         <is>
-          <t>Levantamento Corpo</t>
+          <t>Parachoque + Chapa 2,65</t>
         </is>
       </c>
       <c r="D113" t="n">
@@ -3543,345 +3572,45 @@
       </c>
       <c r="F113" s="1" t="inlineStr">
         <is>
-          <t>000370</t>
+          <t>000378</t>
         </is>
       </c>
     </row>
     <row r="114">
-      <c r="A114" t="inlineStr">
-        <is>
-          <t>PG + ECONOMIA HIBRIDO</t>
-        </is>
-      </c>
-      <c r="B114" t="inlineStr">
-        <is>
-          <t>Solda Mig</t>
-        </is>
-      </c>
-      <c r="C114" t="inlineStr">
-        <is>
-          <t>Chaparia Testeira + Saia + Canaletas</t>
-        </is>
-      </c>
-      <c r="D114" t="n">
-        <v>1</v>
-      </c>
-      <c r="E114" t="n">
-        <v>1000</v>
-      </c>
-      <c r="F114" s="1" t="inlineStr">
-        <is>
-          <t>000371</t>
-        </is>
-      </c>
+      <c r="F114" s="1" t="n"/>
     </row>
     <row r="115">
-      <c r="A115" t="inlineStr">
-        <is>
-          <t>PG + ECONOMIA HIBRIDO</t>
-        </is>
-      </c>
-      <c r="B115" t="inlineStr">
-        <is>
-          <t>Solda Mig</t>
-        </is>
-      </c>
-      <c r="C115" t="inlineStr">
-        <is>
-          <t>Bdj Esquerda Tubo + Mão francesa (inferior)</t>
-        </is>
-      </c>
-      <c r="D115" t="n">
-        <v>4</v>
-      </c>
-      <c r="E115" t="n">
-        <v>4000</v>
-      </c>
-      <c r="F115" s="1" t="inlineStr">
-        <is>
-          <t>001441</t>
-        </is>
-      </c>
+      <c r="F115" s="1" t="n"/>
     </row>
     <row r="116">
-      <c r="A116" t="inlineStr">
-        <is>
-          <t>PG + ECONOMIA HIBRIDO</t>
-        </is>
-      </c>
-      <c r="B116" t="inlineStr">
-        <is>
-          <t>Solda Mig</t>
-        </is>
-      </c>
-      <c r="C116" t="inlineStr">
-        <is>
-          <t>Bdj Direita Tubo + Mão francesa (inferior)</t>
-        </is>
-      </c>
-      <c r="D116" t="n">
-        <v>4</v>
-      </c>
-      <c r="E116" t="n">
-        <v>4000</v>
-      </c>
-      <c r="F116" s="1" t="inlineStr">
-        <is>
-          <t>001442</t>
-        </is>
-      </c>
+      <c r="F116" s="1" t="n"/>
     </row>
     <row r="117">
-      <c r="A117" t="inlineStr">
-        <is>
-          <t>PG + ECONOMIA HIBRIDO</t>
-        </is>
-      </c>
-      <c r="B117" t="inlineStr">
-        <is>
-          <t>Solda Mig</t>
-        </is>
-      </c>
-      <c r="C117" t="inlineStr">
-        <is>
-          <t>Bdj Esquerda Base Tubo + Mão francesa (inferior)</t>
-        </is>
-      </c>
-      <c r="D117" t="n">
-        <v>1</v>
-      </c>
-      <c r="E117" t="n">
-        <v>1000</v>
-      </c>
-      <c r="F117" s="1" t="inlineStr">
-        <is>
-          <t>001443</t>
-        </is>
-      </c>
+      <c r="F117" s="1" t="n"/>
     </row>
     <row r="118">
-      <c r="A118" t="inlineStr">
-        <is>
-          <t>PG + ECONOMIA HIBRIDO</t>
-        </is>
-      </c>
-      <c r="B118" t="inlineStr">
-        <is>
-          <t>Solda Mig</t>
-        </is>
-      </c>
-      <c r="C118" t="inlineStr">
-        <is>
-          <t>Bdj Direita Base Tubo + Mão francesa (inferior)</t>
-        </is>
-      </c>
-      <c r="D118" t="n">
-        <v>1</v>
-      </c>
-      <c r="E118" t="n">
-        <v>1000</v>
-      </c>
-      <c r="F118" s="1" t="inlineStr">
-        <is>
-          <t>001444</t>
-        </is>
-      </c>
+      <c r="F118" s="1" t="n"/>
     </row>
     <row r="119">
-      <c r="A119" t="inlineStr">
-        <is>
-          <t>PG + ECONOMIA HIBRIDO</t>
-        </is>
-      </c>
-      <c r="B119" t="inlineStr">
-        <is>
-          <t>Solda Mig</t>
-        </is>
-      </c>
-      <c r="C119" t="inlineStr">
-        <is>
-          <t>Bdj Esquerda Tubo + Mão francesa (superior)</t>
-        </is>
-      </c>
-      <c r="D119" t="n">
-        <v>4</v>
-      </c>
-      <c r="E119" t="n">
-        <v>4000</v>
-      </c>
-      <c r="F119" s="1" t="inlineStr">
-        <is>
-          <t>001445</t>
-        </is>
-      </c>
+      <c r="F119" s="1" t="n"/>
     </row>
     <row r="120">
-      <c r="A120" t="inlineStr">
-        <is>
-          <t>PG + ECONOMIA HIBRIDO</t>
-        </is>
-      </c>
-      <c r="B120" t="inlineStr">
-        <is>
-          <t>Solda Mig</t>
-        </is>
-      </c>
-      <c r="C120" t="inlineStr">
-        <is>
-          <t>Bdj Direita Tubo + Mão francesa (superior)</t>
-        </is>
-      </c>
-      <c r="D120" t="n">
-        <v>4</v>
-      </c>
-      <c r="E120" t="n">
-        <v>4000</v>
-      </c>
-      <c r="F120" s="1" t="inlineStr">
-        <is>
-          <t>001446</t>
-        </is>
-      </c>
+      <c r="F120" s="1" t="n"/>
     </row>
     <row r="121">
-      <c r="A121" t="inlineStr">
-        <is>
-          <t>PG + ECONOMIA HIBRIDO</t>
-        </is>
-      </c>
-      <c r="B121" t="inlineStr">
-        <is>
-          <t>Solda Mig</t>
-        </is>
-      </c>
-      <c r="C121" t="inlineStr">
-        <is>
-          <t>Bdj Esquerda Base Tubo + Mão francesa (superior)</t>
-        </is>
-      </c>
-      <c r="D121" t="n">
-        <v>1</v>
-      </c>
-      <c r="E121" t="n">
-        <v>1000</v>
-      </c>
-      <c r="F121" s="1" t="inlineStr">
-        <is>
-          <t>001447</t>
-        </is>
-      </c>
+      <c r="F121" s="1" t="n"/>
     </row>
     <row r="122">
-      <c r="A122" t="inlineStr">
-        <is>
-          <t>PG + ECONOMIA HIBRIDO</t>
-        </is>
-      </c>
-      <c r="B122" t="inlineStr">
-        <is>
-          <t>Solda Mig</t>
-        </is>
-      </c>
-      <c r="C122" t="inlineStr">
-        <is>
-          <t>Bdj Direita Base Tubo + Mão francesa (superior)</t>
-        </is>
-      </c>
-      <c r="D122" t="n">
-        <v>1</v>
-      </c>
-      <c r="E122" t="n">
-        <v>1000</v>
-      </c>
-      <c r="F122" s="1" t="inlineStr">
-        <is>
-          <t>001448</t>
-        </is>
-      </c>
+      <c r="F122" s="1" t="n"/>
     </row>
     <row r="123">
-      <c r="A123" t="inlineStr">
-        <is>
-          <t>PG + ECONOMIA HIBRIDO</t>
-        </is>
-      </c>
-      <c r="B123" t="inlineStr">
-        <is>
-          <t>Solda Mig</t>
-        </is>
-      </c>
-      <c r="C123" t="inlineStr">
-        <is>
-          <t>Aramado Toldo</t>
-        </is>
-      </c>
-      <c r="D123" t="n">
-        <v>1</v>
-      </c>
-      <c r="E123" t="n">
-        <v>1000</v>
-      </c>
-      <c r="F123" s="1" t="inlineStr">
-        <is>
-          <t>000376</t>
-        </is>
-      </c>
+      <c r="F123" s="1" t="n"/>
     </row>
     <row r="124">
-      <c r="A124" t="inlineStr">
-        <is>
-          <t>PG + ECONOMIA HIBRIDO</t>
-        </is>
-      </c>
-      <c r="B124" t="inlineStr">
-        <is>
-          <t>Solda Mig</t>
-        </is>
-      </c>
-      <c r="C124" t="inlineStr">
-        <is>
-          <t>Aramado Toldo + Chapa Fixação</t>
-        </is>
-      </c>
-      <c r="D124" t="n">
-        <v>1</v>
-      </c>
-      <c r="E124" t="n">
-        <v>1000</v>
-      </c>
-      <c r="F124" s="1" t="inlineStr">
-        <is>
-          <t>000377</t>
-        </is>
-      </c>
+      <c r="F124" s="1" t="n"/>
     </row>
     <row r="125">
-      <c r="A125" t="inlineStr">
-        <is>
-          <t>PG + ECONOMIA HIBRIDO</t>
-        </is>
-      </c>
-      <c r="B125" t="inlineStr">
-        <is>
-          <t>Solda Mig</t>
-        </is>
-      </c>
-      <c r="C125" t="inlineStr">
-        <is>
-          <t>Parachoque + Chapa 2,65</t>
-        </is>
-      </c>
-      <c r="D125" t="n">
-        <v>1</v>
-      </c>
-      <c r="E125" t="n">
-        <v>1000</v>
-      </c>
-      <c r="F125" s="1" t="inlineStr">
-        <is>
-          <t>000378</t>
-        </is>
-      </c>
+      <c r="F125" s="1" t="n"/>
     </row>
     <row r="126">
       <c r="F126" s="1" t="n"/>
@@ -3891,42 +3620,6 @@
     </row>
     <row r="128">
       <c r="F128" s="1" t="n"/>
-    </row>
-    <row r="129">
-      <c r="F129" s="1" t="n"/>
-    </row>
-    <row r="130">
-      <c r="F130" s="1" t="n"/>
-    </row>
-    <row r="131">
-      <c r="F131" s="1" t="n"/>
-    </row>
-    <row r="132">
-      <c r="F132" s="1" t="n"/>
-    </row>
-    <row r="133">
-      <c r="F133" s="1" t="n"/>
-    </row>
-    <row r="134">
-      <c r="F134" s="1" t="n"/>
-    </row>
-    <row r="135">
-      <c r="F135" s="1" t="n"/>
-    </row>
-    <row r="136">
-      <c r="F136" s="1" t="n"/>
-    </row>
-    <row r="137">
-      <c r="F137" s="1" t="n"/>
-    </row>
-    <row r="138">
-      <c r="F138" s="1" t="n"/>
-    </row>
-    <row r="139">
-      <c r="F139" s="1" t="n"/>
-    </row>
-    <row r="140">
-      <c r="F140" s="1" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Automatiza 114 arquivo(s) de processos no backend
</commit_message>
<xml_diff>
--- a/planilhas/LISTA DE PROCESSO PG + ECO HIBRIDO LADO MENOR.xlsx
+++ b/planilhas/LISTA DE PROCESSO PG + ECO HIBRIDO LADO MENOR.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-105" yWindow="0" windowWidth="14610" windowHeight="15585" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
     <sheet name="Plan1" sheetId="1" state="visible" r:id="rId1"/>
@@ -16,15 +16,11 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="2">
+  <fonts count="1">
     <font>
       <name val="Calibri"/>
       <color theme="1"/>
       <sz val="11"/>
-    </font>
-    <font>
-      <name val="Calibri"/>
-      <sz val="8"/>
     </font>
   </fonts>
   <fills count="2">
@@ -387,7 +383,7 @@
         </is>
       </c>
       <c r="D2">
-        <f>E2/100</f>
+        <f>E2/1000</f>
         <v/>
       </c>
       <c r="E2" t="n">
@@ -416,7 +412,7 @@
         </is>
       </c>
       <c r="D3">
-        <f>E3/100</f>
+        <f>E3/1000</f>
         <v/>
       </c>
       <c r="E3" t="n">
@@ -445,7 +441,7 @@
         </is>
       </c>
       <c r="D4">
-        <f>E4/100</f>
+        <f>E4/1000</f>
         <v/>
       </c>
       <c r="E4" t="n">
@@ -474,7 +470,7 @@
         </is>
       </c>
       <c r="D5">
-        <f>E5/100</f>
+        <f>E5/1000</f>
         <v/>
       </c>
       <c r="E5" t="n">
@@ -503,7 +499,7 @@
         </is>
       </c>
       <c r="D6">
-        <f>E6/100</f>
+        <f>E6/1000</f>
         <v/>
       </c>
       <c r="E6" t="n">
@@ -532,7 +528,7 @@
         </is>
       </c>
       <c r="D7">
-        <f>E7/100</f>
+        <f>E7/1000</f>
         <v/>
       </c>
       <c r="E7" t="n">
@@ -561,7 +557,7 @@
         </is>
       </c>
       <c r="D8">
-        <f>E8/100</f>
+        <f>E8/1000</f>
         <v/>
       </c>
       <c r="E8" t="n">
@@ -590,7 +586,7 @@
         </is>
       </c>
       <c r="D9">
-        <f>E9/100</f>
+        <f>E9/1000</f>
         <v/>
       </c>
       <c r="E9" t="n">
@@ -619,7 +615,7 @@
         </is>
       </c>
       <c r="D10">
-        <f>E10/100</f>
+        <f>E10/1000</f>
         <v/>
       </c>
       <c r="E10" t="n">
@@ -648,7 +644,7 @@
         </is>
       </c>
       <c r="D11">
-        <f>E11/100</f>
+        <f>E11/1000</f>
         <v/>
       </c>
       <c r="E11" t="n">
@@ -677,7 +673,7 @@
         </is>
       </c>
       <c r="D12">
-        <f>E12/100</f>
+        <f>E12/1000</f>
         <v/>
       </c>
       <c r="E12" t="n">
@@ -706,7 +702,7 @@
         </is>
       </c>
       <c r="D13">
-        <f>E13/100</f>
+        <f>E13/1000</f>
         <v/>
       </c>
       <c r="E13" t="n">
@@ -735,7 +731,7 @@
         </is>
       </c>
       <c r="D14">
-        <f>E14/100</f>
+        <f>E14/1000</f>
         <v/>
       </c>
       <c r="E14" t="n">
@@ -764,7 +760,7 @@
         </is>
       </c>
       <c r="D15">
-        <f>E15/100</f>
+        <f>E15/1000</f>
         <v/>
       </c>
       <c r="E15" t="n">
@@ -793,7 +789,7 @@
         </is>
       </c>
       <c r="D16">
-        <f>E16/100</f>
+        <f>E16/1000</f>
         <v/>
       </c>
       <c r="E16" t="n">
@@ -822,7 +818,7 @@
         </is>
       </c>
       <c r="D17">
-        <f>E17/100</f>
+        <f>E17/1000</f>
         <v/>
       </c>
       <c r="E17" t="n">
@@ -851,7 +847,7 @@
         </is>
       </c>
       <c r="D18">
-        <f>E18/100</f>
+        <f>E18/1000</f>
         <v/>
       </c>
       <c r="E18" t="n">
@@ -880,7 +876,7 @@
         </is>
       </c>
       <c r="D19">
-        <f>E19/100</f>
+        <f>E19/1000</f>
         <v/>
       </c>
       <c r="E19" t="n">
@@ -909,7 +905,7 @@
         </is>
       </c>
       <c r="D20">
-        <f>E20/100</f>
+        <f>E20/1000</f>
         <v/>
       </c>
       <c r="E20" t="n">
@@ -938,7 +934,7 @@
         </is>
       </c>
       <c r="D21">
-        <f>E21/100</f>
+        <f>E21/1000</f>
         <v/>
       </c>
       <c r="E21" t="n">
@@ -967,7 +963,7 @@
         </is>
       </c>
       <c r="D22">
-        <f>E22/100</f>
+        <f>E22/1000</f>
         <v/>
       </c>
       <c r="E22" t="n">
@@ -996,7 +992,7 @@
         </is>
       </c>
       <c r="D23">
-        <f>E23/100</f>
+        <f>E23/1000</f>
         <v/>
       </c>
       <c r="E23" t="n">
@@ -1025,7 +1021,7 @@
         </is>
       </c>
       <c r="D24">
-        <f>E24/100</f>
+        <f>E24/1000</f>
         <v/>
       </c>
       <c r="E24" t="n">
@@ -1054,7 +1050,7 @@
         </is>
       </c>
       <c r="D25">
-        <f>E25/100</f>
+        <f>E25/1000</f>
         <v/>
       </c>
       <c r="E25" t="n">
@@ -1083,7 +1079,7 @@
         </is>
       </c>
       <c r="D26">
-        <f>E26/100</f>
+        <f>E26/1000</f>
         <v/>
       </c>
       <c r="E26" t="n">
@@ -1112,7 +1108,7 @@
         </is>
       </c>
       <c r="D27">
-        <f>E27/100</f>
+        <f>E27/1000</f>
         <v/>
       </c>
       <c r="E27" t="n">
@@ -1141,7 +1137,7 @@
         </is>
       </c>
       <c r="D28">
-        <f>E28/100</f>
+        <f>E28/1000</f>
         <v/>
       </c>
       <c r="E28" t="n">
@@ -1170,7 +1166,7 @@
         </is>
       </c>
       <c r="D29">
-        <f>E29/100</f>
+        <f>E29/1000</f>
         <v/>
       </c>
       <c r="E29" t="n">
@@ -1199,7 +1195,7 @@
         </is>
       </c>
       <c r="D30">
-        <f>E30/100</f>
+        <f>E30/1000</f>
         <v/>
       </c>
       <c r="E30" t="n">
@@ -1228,7 +1224,7 @@
         </is>
       </c>
       <c r="D31">
-        <f>E31/100</f>
+        <f>E31/1000</f>
         <v/>
       </c>
       <c r="E31" t="n">
@@ -1464,7 +1460,7 @@
         <v/>
       </c>
       <c r="E39" t="n">
-        <v>57</v>
+        <v>54</v>
       </c>
       <c r="F39" s="1" t="inlineStr">
         <is>
@@ -1522,7 +1518,7 @@
         <v/>
       </c>
       <c r="E41" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="F41" s="1" t="inlineStr">
         <is>
@@ -1580,7 +1576,7 @@
         <v/>
       </c>
       <c r="E43" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F43" s="1" t="inlineStr">
         <is>
@@ -1609,7 +1605,7 @@
         <v/>
       </c>
       <c r="E44" t="n">
-        <v>10</v>
+        <v>3</v>
       </c>
       <c r="F44" s="1" t="inlineStr">
         <is>
@@ -1638,7 +1634,7 @@
         <v/>
       </c>
       <c r="E45" t="n">
-        <v>11</v>
+        <v>1</v>
       </c>
       <c r="F45" s="1" t="inlineStr">
         <is>
@@ -1667,7 +1663,7 @@
         <v/>
       </c>
       <c r="E46" t="n">
-        <v>1</v>
+        <v>9</v>
       </c>
       <c r="F46" s="1" t="inlineStr">
         <is>
@@ -1696,7 +1692,7 @@
         <v/>
       </c>
       <c r="E47" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="F47" s="1" t="inlineStr">
         <is>
@@ -1783,7 +1779,7 @@
         <v/>
       </c>
       <c r="E50" t="n">
-        <v>79</v>
+        <v>30</v>
       </c>
       <c r="F50" s="1" t="inlineStr">
         <is>
@@ -1812,7 +1808,7 @@
         <v/>
       </c>
       <c r="E51" t="n">
-        <v>247</v>
+        <v>248</v>
       </c>
       <c r="F51" s="1" t="inlineStr">
         <is>
@@ -1841,7 +1837,7 @@
         <v/>
       </c>
       <c r="E52" t="n">
-        <v>2</v>
+        <v>10</v>
       </c>
       <c r="F52" s="1" t="inlineStr">
         <is>
@@ -1870,7 +1866,7 @@
         <v/>
       </c>
       <c r="E53" t="n">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="F53" s="1" t="inlineStr">
         <is>
@@ -1899,7 +1895,7 @@
         <v/>
       </c>
       <c r="E54" t="n">
-        <v>1</v>
+        <v>37</v>
       </c>
       <c r="F54" s="1" t="inlineStr">
         <is>
@@ -2127,7 +2123,7 @@
         </is>
       </c>
       <c r="D62">
-        <f>E62/1700</f>
+        <f>E62/1000</f>
         <v/>
       </c>
       <c r="E62" t="n">
@@ -2156,7 +2152,7 @@
         </is>
       </c>
       <c r="D63">
-        <f>E63/1700</f>
+        <f>E63/1000</f>
         <v/>
       </c>
       <c r="E63" t="n">

</xml_diff>